<commit_message>
🔄 Auto-collect traffic data: 2026-09-29 10:09 AM IST
</commit_message>
<xml_diff>
--- a/output/excel/Metro_vs_Car_Data_2026-09-29_Tue.xlsx
+++ b/output/excel/Metro_vs_Car_Data_2026-09-29_Tue.xlsx
@@ -5,14 +5,15 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="All Periods Combined" state="visible" r:id="rId5"/>
+    <sheet sheetId="2" name="10_00 AM" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="All Periods Combined" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1614" uniqueCount="457">
   <si>
     <t>Date</t>
   </si>
@@ -122,7 +123,7 @@
     <t>12:00 AM</t>
   </si>
   <si>
-    <t>Monday (Weekday) - Night Off-Peak</t>
+    <t>Tuesday (Weekday) - Night Off-Peak</t>
   </si>
   <si>
     <t>Blue Line</t>
@@ -824,6 +825,513 @@
     <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/12_00_AM/MC-24/car.jpg</t>
   </si>
   <si>
+    <t>9/29/2026, 10:02:45 AM</t>
+  </si>
+  <si>
+    <t>10:00 AM</t>
+  </si>
+  <si>
+    <t>Tuesday (Weekday) - Morning Peak</t>
+  </si>
+  <si>
+    <t> | 28 min | 10:00 AM—10:28 AM | Blue Line | 10:00 AM from Dakshineswar | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 51 min | 12.2 km | via Barrackpore Trunk Rd | Fastest route, despite slowdown on SH 1 causing 9-min delay | Details | Preview</t>
+  </si>
+  <si>
+    <t>23 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.82x</t>
+  </si>
+  <si>
+    <t>45.1% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-01/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-01/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:03:02 AM</t>
+  </si>
+  <si>
+    <t> | 28 min | 10:03 AM—10:31 AM | Blue Line | 10:03 AM from Shahid Khudiram | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 59 min | 15.1 km | via Netaji Subhas Chandra Bose Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>31 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.11x</t>
+  </si>
+  <si>
+    <t>52.5% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-02/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-02/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:03:19 AM</t>
+  </si>
+  <si>
+    <t> | 7 min | 10:05 AM—10:12 AM | Blue Line | 10:05 AM from Shyambazar | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t> | 17 min | 3.5 km | via Belgachia Rd/Khudiram Bose Sarani | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>10 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.43x</t>
+  </si>
+  <si>
+    <t>58.8% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-03/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-03/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:03:35 AM</t>
+  </si>
+  <si>
+    <t> | 11 min | 10:05 AM—10:16 AM | Blue Line | 10:05 AM from Shyambazar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 23 min | 5.2 km | via Jatindra Mohan Ave and Central Ave/Chittaranjan Ave | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>2.09x</t>
+  </si>
+  <si>
+    <t>52.2% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-04/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-04/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:03:53 AM</t>
+  </si>
+  <si>
+    <t> | 11 min | 10:02 AM—10:13 AM | Blue Line | 10:02 AM from Kalighat | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 20 min | 5.6 km | via Shyama Prasad Mukherjee Rd and Ashutosh Mukherjee Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>45.0% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-05/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-05/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:04:09 AM</t>
+  </si>
+  <si>
+    <t> | 12 min | 10:00 AM—10:12 AM | Blue Line | 10:00 AM from Dakshineswar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 30 min | 7.0 km | via Barrackpore Trunk Rd | Fastest route, despite slowdown on SH 1 causing 9-min delay | Details | Preview</t>
+  </si>
+  <si>
+    <t>18 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.50x</t>
+  </si>
+  <si>
+    <t>60.0% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-06/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-06/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:04:27 AM</t>
+  </si>
+  <si>
+    <t> | 17 min | 10:04 AM—10:21 AM | Blue Line | 10:04 AM from Esplanade | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 31 min | 7.8 km | via Chowringee Rd/Jawaharlal Nehru Rd and Ashutosh Mukherjee Rd | Fastest route, despite heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>14 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>45.2% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-07/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-07/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:04:44 AM</t>
+  </si>
+  <si>
+    <t> | 15 min | 10:03 AM—10:18 AM | Blue Line | 10:03 AM from Mahanayak Uttam Kumar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 27 min | 6.4 km | via Netaji Subhas Chandra Bose Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.80x</t>
+  </si>
+  <si>
+    <t>44.4% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-08/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-08/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:05:02 AM</t>
+  </si>
+  <si>
+    <t> | 16 min | 10:00 AM—10:16 AM | Blue Line | 10:00 AM from Dumdum | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 38 min | 8.6 km | via Jessore Rd and Lock Gate Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>22 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.38x</t>
+  </si>
+  <si>
+    <t>57.9% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-09/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-09/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:05:20 AM</t>
+  </si>
+  <si>
+    <t> | 30 min | 10:02 AM—10:32 AM | Green Line | 10:02 AM from Howrah | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t> | 51 min | 12.4 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>21 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.70x</t>
+  </si>
+  <si>
+    <t>41.2% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-10/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-10/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:05:37 AM</t>
+  </si>
+  <si>
+    <t> | 21 min | 10:05 AM—10:26 AM | Green Line | 10:05 AM from Sealdah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 35 min | 7.8 km | via Beleghata Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-11/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-11/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:05:54 AM</t>
+  </si>
+  <si>
+    <t> | 9 min | 10:02 AM—10:11 AM | Green Line | 10:02 AM from Howrah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 33 min | 7.2 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>24 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>3.67x</t>
+  </si>
+  <si>
+    <t>72.7% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-12/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-12/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:06:11 AM</t>
+  </si>
+  <si>
+    <t> | 18 min | 10:02 AM—10:20 AM | Green Line | 10:02 AM from Phoolbagan | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 22 min | 4.9 km | via Narkeldanga Main Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.22x</t>
+  </si>
+  <si>
+    <t>18.2% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-13/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-13/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:06:28 AM</t>
+  </si>
+  <si>
+    <t> | 12 min | 10:02 AM—10:14 AM | Green Line | 10:02 AM from Howrah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 34 min | 7.6 km | via Kali Krishna Tagore St | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>2.83x</t>
+  </si>
+  <si>
+    <t>64.7% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-14/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-14/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:06:45 AM</t>
+  </si>
+  <si>
+    <t> | 25 min | 10:01 AM—10:26 AM | Green Line | 10:01 AM from Esplanade | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t> | 46 min | 15.7 km | via Circus Ave | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.84x</t>
+  </si>
+  <si>
+    <t>45.7% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-15/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-15/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:07:01 AM</t>
+  </si>
+  <si>
+    <t> | 23 min | 10:20 AM—10:43 AM | Orange Line | 10:20 AM from Kavi Subhash | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 30 min | 10.0 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>7 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.30x</t>
+  </si>
+  <si>
+    <t>23.3% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-16/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-16/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:07:19 AM</t>
+  </si>
+  <si>
+    <t> | 12 min | 10:06 AM—10:18 AM | Orange Line | 10:06 AM from Hemanta Mukhopadhyay | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t> | 14 min | 4.4 km | via Bangaon - Kulpi Rd/Biswa Bangla Sarani/Eastern Metropolitan Bypass/Thakurnagar - Panchpota Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-17/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-17/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:07:37 AM</t>
+  </si>
+  <si>
+    <t> | 19 min | 10:20 AM—10:39 AM | Orange Line | 10:20 AM from Kavi Subhash | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 28 min | 8.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.47x</t>
+  </si>
+  <si>
+    <t>32.1% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-18/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-18/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:07:55 AM</t>
+  </si>
+  <si>
+    <t> | 17 min | 10:14 AM—10:31 AM | Purple Line | 10:14 AM from Joka | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 27 min | 7.8 km | via NH 12 | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.59x</t>
+  </si>
+  <si>
+    <t>37.0% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-19/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-19/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:08:11 AM</t>
+  </si>
+  <si>
+    <t> | 9 min | 10:01 AM—10:10 AM | Purple Line | 10:01 AM from Behala Chowrasta | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t> | 13 min | 3.7 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.44x</t>
+  </si>
+  <si>
+    <t>30.8% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-20/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-20/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:08:28 AM</t>
+  </si>
+  <si>
+    <t> | 8 min | 10:14 AM—10:22 AM | Purple Line | 10:14 AM from Joka | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t> | 14 min | 4.1 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-21/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-21/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:08:45 AM</t>
+  </si>
+  <si>
+    <t> | 14 min | 10:14 AM—10:28 AM | Purple Line | 10:14 AM from Joka | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 23 min | 6.5 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.64x</t>
+  </si>
+  <si>
+    <t>39.1% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-22/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-22/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:09:02 AM</t>
+  </si>
+  <si>
+    <t> | 6 min | 10:01 AM—10:07 AM | Purple Line | 10:01 AM from Behala Chowrasta | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t> | 9 min | 2.4 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.50x</t>
+  </si>
+  <si>
+    <t>33.3% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-23/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-23/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 10:09:19 AM</t>
+  </si>
+  <si>
+    <t> | 3 min | 10:07 AM—10:10 AM | Purple Line | 10:07 AM from Taratala | ₹5.00 | Details</t>
+  </si>
+  <si>
+    <t> | 3 min | 1.3 km | via NH 12 | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-24/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-24/car.jpg</t>
+  </si>
+  <si>
     <t>12:00 AM Scraped At</t>
   </si>
   <si>
@@ -849,6 +1357,33 @@
   </si>
   <si>
     <t>12:00 AM Savings (%)</t>
+  </si>
+  <si>
+    <t>10:00 AM Scraped At</t>
+  </si>
+  <si>
+    <t>10:00 AM Actual Metro</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro Walk</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro (min)</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro Route</t>
+  </si>
+  <si>
+    <t>10:00 AM Metro Raw Details</t>
+  </si>
+  <si>
+    <t>10:00 AM Car (min)</t>
+  </si>
+  <si>
+    <t>10:00 AM Faster Mode</t>
+  </si>
+  <si>
+    <t>10:00 AM Savings (%)</t>
   </si>
 </sst>
 </file>
@@ -3392,10 +3927,2147 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>270</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2">
+        <v>15</v>
+      </c>
+      <c r="J2">
+        <v>12.2</v>
+      </c>
+      <c r="K2" t="s">
+        <v>271</v>
+      </c>
+      <c r="L2" t="s">
+        <v>272</v>
+      </c>
+      <c r="M2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2">
+        <v>28</v>
+      </c>
+      <c r="P2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>273</v>
+      </c>
+      <c r="R2">
+        <v>51</v>
+      </c>
+      <c r="S2" t="s">
+        <v>274</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="U2" t="s">
+        <v>276</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W2" t="s">
+        <v>277</v>
+      </c>
+      <c r="X2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>278</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>280</v>
+      </c>
+      <c r="D3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3">
+        <v>14.9</v>
+      </c>
+      <c r="J3">
+        <v>15.1</v>
+      </c>
+      <c r="K3" t="s">
+        <v>271</v>
+      </c>
+      <c r="L3" t="s">
+        <v>272</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3">
+        <v>28</v>
+      </c>
+      <c r="P3" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>281</v>
+      </c>
+      <c r="R3">
+        <v>59</v>
+      </c>
+      <c r="S3" t="s">
+        <v>282</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="U3" t="s">
+        <v>284</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W3" t="s">
+        <v>285</v>
+      </c>
+      <c r="X3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>286</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>288</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I4">
+        <v>3.8</v>
+      </c>
+      <c r="J4">
+        <v>3.5</v>
+      </c>
+      <c r="K4" t="s">
+        <v>271</v>
+      </c>
+      <c r="L4" t="s">
+        <v>272</v>
+      </c>
+      <c r="M4" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4">
+        <v>7</v>
+      </c>
+      <c r="P4" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>289</v>
+      </c>
+      <c r="R4">
+        <v>17</v>
+      </c>
+      <c r="S4" t="s">
+        <v>290</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="U4" t="s">
+        <v>292</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W4" t="s">
+        <v>293</v>
+      </c>
+      <c r="X4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>294</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>296</v>
+      </c>
+      <c r="D5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5">
+        <v>5.1</v>
+      </c>
+      <c r="J5">
+        <v>5.2</v>
+      </c>
+      <c r="K5" t="s">
+        <v>271</v>
+      </c>
+      <c r="L5" t="s">
+        <v>272</v>
+      </c>
+      <c r="M5" t="s">
+        <v>37</v>
+      </c>
+      <c r="N5" t="s">
+        <v>38</v>
+      </c>
+      <c r="O5">
+        <v>11</v>
+      </c>
+      <c r="P5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>297</v>
+      </c>
+      <c r="R5">
+        <v>23</v>
+      </c>
+      <c r="S5" t="s">
+        <v>298</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="U5" t="s">
+        <v>299</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W5" t="s">
+        <v>300</v>
+      </c>
+      <c r="X5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>301</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>303</v>
+      </c>
+      <c r="D6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6">
+        <v>5.2</v>
+      </c>
+      <c r="J6">
+        <v>5.6</v>
+      </c>
+      <c r="K6" t="s">
+        <v>271</v>
+      </c>
+      <c r="L6" t="s">
+        <v>272</v>
+      </c>
+      <c r="M6" t="s">
+        <v>37</v>
+      </c>
+      <c r="N6" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6">
+        <v>11</v>
+      </c>
+      <c r="P6" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>304</v>
+      </c>
+      <c r="R6">
+        <v>20</v>
+      </c>
+      <c r="S6" t="s">
+        <v>305</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="U6" t="s">
+        <v>276</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W6" t="s">
+        <v>306</v>
+      </c>
+      <c r="X6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>307</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>309</v>
+      </c>
+      <c r="D7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I7">
+        <v>6.2</v>
+      </c>
+      <c r="J7">
+        <v>7</v>
+      </c>
+      <c r="K7" t="s">
+        <v>271</v>
+      </c>
+      <c r="L7" t="s">
+        <v>272</v>
+      </c>
+      <c r="M7" t="s">
+        <v>37</v>
+      </c>
+      <c r="N7" t="s">
+        <v>38</v>
+      </c>
+      <c r="O7">
+        <v>12</v>
+      </c>
+      <c r="P7" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>310</v>
+      </c>
+      <c r="R7">
+        <v>30</v>
+      </c>
+      <c r="S7" t="s">
+        <v>311</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="U7" t="s">
+        <v>313</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W7" t="s">
+        <v>314</v>
+      </c>
+      <c r="X7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>315</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>317</v>
+      </c>
+      <c r="D8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" t="s">
+        <v>100</v>
+      </c>
+      <c r="I8">
+        <v>7.8</v>
+      </c>
+      <c r="J8">
+        <v>7.8</v>
+      </c>
+      <c r="K8" t="s">
+        <v>271</v>
+      </c>
+      <c r="L8" t="s">
+        <v>272</v>
+      </c>
+      <c r="M8" t="s">
+        <v>37</v>
+      </c>
+      <c r="N8" t="s">
+        <v>38</v>
+      </c>
+      <c r="O8">
+        <v>17</v>
+      </c>
+      <c r="P8" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>318</v>
+      </c>
+      <c r="R8">
+        <v>31</v>
+      </c>
+      <c r="S8" t="s">
+        <v>319</v>
+      </c>
+      <c r="T8" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="U8" t="s">
+        <v>276</v>
+      </c>
+      <c r="V8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W8" t="s">
+        <v>321</v>
+      </c>
+      <c r="X8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>322</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>324</v>
+      </c>
+      <c r="D9" t="s">
+        <v>109</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" t="s">
+        <v>100</v>
+      </c>
+      <c r="H9" t="s">
+        <v>110</v>
+      </c>
+      <c r="I9">
+        <v>7.1</v>
+      </c>
+      <c r="J9">
+        <v>6.4</v>
+      </c>
+      <c r="K9" t="s">
+        <v>271</v>
+      </c>
+      <c r="L9" t="s">
+        <v>272</v>
+      </c>
+      <c r="M9" t="s">
+        <v>37</v>
+      </c>
+      <c r="N9" t="s">
+        <v>38</v>
+      </c>
+      <c r="O9">
+        <v>15</v>
+      </c>
+      <c r="P9" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>325</v>
+      </c>
+      <c r="R9">
+        <v>27</v>
+      </c>
+      <c r="S9" t="s">
+        <v>326</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="U9" t="s">
+        <v>327</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W9" t="s">
+        <v>328</v>
+      </c>
+      <c r="X9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>329</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>331</v>
+      </c>
+      <c r="D10" t="s">
+        <v>120</v>
+      </c>
+      <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10">
+        <v>8.8</v>
+      </c>
+      <c r="J10">
+        <v>8.6</v>
+      </c>
+      <c r="K10" t="s">
+        <v>271</v>
+      </c>
+      <c r="L10" t="s">
+        <v>272</v>
+      </c>
+      <c r="M10" t="s">
+        <v>37</v>
+      </c>
+      <c r="N10" t="s">
+        <v>38</v>
+      </c>
+      <c r="O10">
+        <v>16</v>
+      </c>
+      <c r="P10" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>332</v>
+      </c>
+      <c r="R10">
+        <v>38</v>
+      </c>
+      <c r="S10" t="s">
+        <v>333</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="U10" t="s">
+        <v>335</v>
+      </c>
+      <c r="V10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W10" t="s">
+        <v>336</v>
+      </c>
+      <c r="X10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>337</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>339</v>
+      </c>
+      <c r="D11" t="s">
+        <v>129</v>
+      </c>
+      <c r="E11" t="s">
+        <v>130</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>131</v>
+      </c>
+      <c r="H11" t="s">
+        <v>132</v>
+      </c>
+      <c r="I11">
+        <v>14.2</v>
+      </c>
+      <c r="J11">
+        <v>12.4</v>
+      </c>
+      <c r="K11" t="s">
+        <v>271</v>
+      </c>
+      <c r="L11" t="s">
+        <v>272</v>
+      </c>
+      <c r="M11" t="s">
+        <v>133</v>
+      </c>
+      <c r="N11" t="s">
+        <v>38</v>
+      </c>
+      <c r="O11">
+        <v>30</v>
+      </c>
+      <c r="P11" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>340</v>
+      </c>
+      <c r="R11">
+        <v>51</v>
+      </c>
+      <c r="S11" t="s">
+        <v>341</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="U11" t="s">
+        <v>343</v>
+      </c>
+      <c r="V11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W11" t="s">
+        <v>344</v>
+      </c>
+      <c r="X11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>345</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>347</v>
+      </c>
+      <c r="D12" t="s">
+        <v>143</v>
+      </c>
+      <c r="E12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" t="s">
+        <v>144</v>
+      </c>
+      <c r="H12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I12">
+        <v>8.6</v>
+      </c>
+      <c r="J12">
+        <v>7.8</v>
+      </c>
+      <c r="K12" t="s">
+        <v>271</v>
+      </c>
+      <c r="L12" t="s">
+        <v>272</v>
+      </c>
+      <c r="M12" t="s">
+        <v>133</v>
+      </c>
+      <c r="N12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O12">
+        <v>21</v>
+      </c>
+      <c r="P12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>348</v>
+      </c>
+      <c r="R12">
+        <v>35</v>
+      </c>
+      <c r="S12" t="s">
+        <v>349</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="U12" t="s">
+        <v>94</v>
+      </c>
+      <c r="V12" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W12" t="s">
+        <v>95</v>
+      </c>
+      <c r="X12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>350</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>352</v>
+      </c>
+      <c r="D13" t="s">
+        <v>153</v>
+      </c>
+      <c r="E13" t="s">
+        <v>130</v>
+      </c>
+      <c r="F13" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" t="s">
+        <v>131</v>
+      </c>
+      <c r="H13" t="s">
+        <v>144</v>
+      </c>
+      <c r="I13">
+        <v>5.6</v>
+      </c>
+      <c r="J13">
+        <v>7.2</v>
+      </c>
+      <c r="K13" t="s">
+        <v>271</v>
+      </c>
+      <c r="L13" t="s">
+        <v>272</v>
+      </c>
+      <c r="M13" t="s">
+        <v>133</v>
+      </c>
+      <c r="N13" t="s">
+        <v>38</v>
+      </c>
+      <c r="O13">
+        <v>9</v>
+      </c>
+      <c r="P13" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>353</v>
+      </c>
+      <c r="R13">
+        <v>33</v>
+      </c>
+      <c r="S13" t="s">
+        <v>354</v>
+      </c>
+      <c r="T13" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="U13" t="s">
+        <v>356</v>
+      </c>
+      <c r="V13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W13" t="s">
+        <v>357</v>
+      </c>
+      <c r="X13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>358</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>360</v>
+      </c>
+      <c r="D14" t="s">
+        <v>162</v>
+      </c>
+      <c r="E14" t="s">
+        <v>130</v>
+      </c>
+      <c r="F14" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" t="s">
+        <v>163</v>
+      </c>
+      <c r="H14" t="s">
+        <v>132</v>
+      </c>
+      <c r="I14">
+        <v>6.6</v>
+      </c>
+      <c r="J14">
+        <v>4.9</v>
+      </c>
+      <c r="K14" t="s">
+        <v>271</v>
+      </c>
+      <c r="L14" t="s">
+        <v>272</v>
+      </c>
+      <c r="M14" t="s">
+        <v>133</v>
+      </c>
+      <c r="N14" t="s">
+        <v>38</v>
+      </c>
+      <c r="O14">
+        <v>18</v>
+      </c>
+      <c r="P14" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>361</v>
+      </c>
+      <c r="R14">
+        <v>22</v>
+      </c>
+      <c r="S14" t="s">
+        <v>362</v>
+      </c>
+      <c r="T14" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="U14" t="s">
+        <v>363</v>
+      </c>
+      <c r="V14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W14" t="s">
+        <v>364</v>
+      </c>
+      <c r="X14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>365</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>367</v>
+      </c>
+      <c r="D15" t="s">
+        <v>172</v>
+      </c>
+      <c r="E15" t="s">
+        <v>130</v>
+      </c>
+      <c r="F15" t="s">
+        <v>60</v>
+      </c>
+      <c r="G15" t="s">
+        <v>131</v>
+      </c>
+      <c r="H15" t="s">
+        <v>163</v>
+      </c>
+      <c r="I15">
+        <v>7.7</v>
+      </c>
+      <c r="J15">
+        <v>7.6</v>
+      </c>
+      <c r="K15" t="s">
+        <v>271</v>
+      </c>
+      <c r="L15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M15" t="s">
+        <v>133</v>
+      </c>
+      <c r="N15" t="s">
+        <v>38</v>
+      </c>
+      <c r="O15">
+        <v>12</v>
+      </c>
+      <c r="P15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>368</v>
+      </c>
+      <c r="R15">
+        <v>34</v>
+      </c>
+      <c r="S15" t="s">
+        <v>369</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="U15" t="s">
+        <v>370</v>
+      </c>
+      <c r="V15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W15" t="s">
+        <v>371</v>
+      </c>
+      <c r="X15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>372</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>374</v>
+      </c>
+      <c r="D16" t="s">
+        <v>181</v>
+      </c>
+      <c r="E16" t="s">
+        <v>130</v>
+      </c>
+      <c r="F16" t="s">
+        <v>60</v>
+      </c>
+      <c r="G16" t="s">
+        <v>34</v>
+      </c>
+      <c r="H16" t="s">
+        <v>132</v>
+      </c>
+      <c r="I16">
+        <v>11.3</v>
+      </c>
+      <c r="J16">
+        <v>15.7</v>
+      </c>
+      <c r="K16" t="s">
+        <v>271</v>
+      </c>
+      <c r="L16" t="s">
+        <v>272</v>
+      </c>
+      <c r="M16" t="s">
+        <v>133</v>
+      </c>
+      <c r="N16" t="s">
+        <v>38</v>
+      </c>
+      <c r="O16">
+        <v>25</v>
+      </c>
+      <c r="P16" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>375</v>
+      </c>
+      <c r="R16">
+        <v>46</v>
+      </c>
+      <c r="S16" t="s">
+        <v>376</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="U16" t="s">
+        <v>377</v>
+      </c>
+      <c r="V16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W16" t="s">
+        <v>378</v>
+      </c>
+      <c r="X16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>379</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>381</v>
+      </c>
+      <c r="D17" t="s">
+        <v>190</v>
+      </c>
+      <c r="E17" t="s">
+        <v>191</v>
+      </c>
+      <c r="F17" t="s">
+        <v>32</v>
+      </c>
+      <c r="G17" t="s">
+        <v>110</v>
+      </c>
+      <c r="H17" t="s">
+        <v>192</v>
+      </c>
+      <c r="I17">
+        <v>9.8</v>
+      </c>
+      <c r="J17">
+        <v>10</v>
+      </c>
+      <c r="K17" t="s">
+        <v>271</v>
+      </c>
+      <c r="L17" t="s">
+        <v>272</v>
+      </c>
+      <c r="M17" t="s">
+        <v>193</v>
+      </c>
+      <c r="N17" t="s">
+        <v>38</v>
+      </c>
+      <c r="O17">
+        <v>23</v>
+      </c>
+      <c r="P17" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>382</v>
+      </c>
+      <c r="R17">
+        <v>30</v>
+      </c>
+      <c r="S17" t="s">
+        <v>383</v>
+      </c>
+      <c r="T17" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="U17" t="s">
+        <v>385</v>
+      </c>
+      <c r="V17" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W17" t="s">
+        <v>386</v>
+      </c>
+      <c r="X17" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>387</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" t="s">
+        <v>389</v>
+      </c>
+      <c r="D18" t="s">
+        <v>202</v>
+      </c>
+      <c r="E18" t="s">
+        <v>191</v>
+      </c>
+      <c r="F18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H18" t="s">
+        <v>192</v>
+      </c>
+      <c r="I18">
+        <v>5.9</v>
+      </c>
+      <c r="J18">
+        <v>4.4</v>
+      </c>
+      <c r="K18" t="s">
+        <v>271</v>
+      </c>
+      <c r="L18" t="s">
+        <v>272</v>
+      </c>
+      <c r="M18" t="s">
+        <v>193</v>
+      </c>
+      <c r="N18" t="s">
+        <v>38</v>
+      </c>
+      <c r="O18">
+        <v>12</v>
+      </c>
+      <c r="P18" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>390</v>
+      </c>
+      <c r="R18">
+        <v>14</v>
+      </c>
+      <c r="S18" t="s">
+        <v>391</v>
+      </c>
+      <c r="T18" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="U18" t="s">
+        <v>258</v>
+      </c>
+      <c r="V18" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W18" t="s">
+        <v>259</v>
+      </c>
+      <c r="X18" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>392</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>394</v>
+      </c>
+      <c r="D19" t="s">
+        <v>210</v>
+      </c>
+      <c r="E19" t="s">
+        <v>191</v>
+      </c>
+      <c r="F19" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" t="s">
+        <v>110</v>
+      </c>
+      <c r="H19" t="s">
+        <v>211</v>
+      </c>
+      <c r="I19">
+        <v>8.9</v>
+      </c>
+      <c r="J19">
+        <v>8.8</v>
+      </c>
+      <c r="K19" t="s">
+        <v>271</v>
+      </c>
+      <c r="L19" t="s">
+        <v>272</v>
+      </c>
+      <c r="M19" t="s">
+        <v>193</v>
+      </c>
+      <c r="N19" t="s">
+        <v>38</v>
+      </c>
+      <c r="O19">
+        <v>19</v>
+      </c>
+      <c r="P19" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>395</v>
+      </c>
+      <c r="R19">
+        <v>28</v>
+      </c>
+      <c r="S19" t="s">
+        <v>396</v>
+      </c>
+      <c r="T19" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="U19" t="s">
+        <v>397</v>
+      </c>
+      <c r="V19" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W19" t="s">
+        <v>398</v>
+      </c>
+      <c r="X19" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>399</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" t="s">
+        <v>401</v>
+      </c>
+      <c r="D20" t="s">
+        <v>219</v>
+      </c>
+      <c r="E20" t="s">
+        <v>220</v>
+      </c>
+      <c r="F20" t="s">
+        <v>32</v>
+      </c>
+      <c r="G20" t="s">
+        <v>221</v>
+      </c>
+      <c r="H20" t="s">
+        <v>222</v>
+      </c>
+      <c r="I20">
+        <v>7.9</v>
+      </c>
+      <c r="J20">
+        <v>7.8</v>
+      </c>
+      <c r="K20" t="s">
+        <v>271</v>
+      </c>
+      <c r="L20" t="s">
+        <v>272</v>
+      </c>
+      <c r="M20" t="s">
+        <v>223</v>
+      </c>
+      <c r="N20" t="s">
+        <v>38</v>
+      </c>
+      <c r="O20">
+        <v>17</v>
+      </c>
+      <c r="P20" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>402</v>
+      </c>
+      <c r="R20">
+        <v>27</v>
+      </c>
+      <c r="S20" t="s">
+        <v>403</v>
+      </c>
+      <c r="T20" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="U20" t="s">
+        <v>404</v>
+      </c>
+      <c r="V20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W20" t="s">
+        <v>405</v>
+      </c>
+      <c r="X20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>406</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" t="s">
+        <v>408</v>
+      </c>
+      <c r="D21" t="s">
+        <v>229</v>
+      </c>
+      <c r="E21" t="s">
+        <v>220</v>
+      </c>
+      <c r="F21" t="s">
+        <v>60</v>
+      </c>
+      <c r="G21" t="s">
+        <v>230</v>
+      </c>
+      <c r="H21" t="s">
+        <v>222</v>
+      </c>
+      <c r="I21">
+        <v>3.7</v>
+      </c>
+      <c r="J21">
+        <v>3.7</v>
+      </c>
+      <c r="K21" t="s">
+        <v>271</v>
+      </c>
+      <c r="L21" t="s">
+        <v>272</v>
+      </c>
+      <c r="M21" t="s">
+        <v>223</v>
+      </c>
+      <c r="N21" t="s">
+        <v>38</v>
+      </c>
+      <c r="O21">
+        <v>9</v>
+      </c>
+      <c r="P21" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>409</v>
+      </c>
+      <c r="R21">
+        <v>13</v>
+      </c>
+      <c r="S21" t="s">
+        <v>410</v>
+      </c>
+      <c r="T21" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="U21" t="s">
+        <v>411</v>
+      </c>
+      <c r="V21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W21" t="s">
+        <v>412</v>
+      </c>
+      <c r="X21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>413</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" t="s">
+        <v>415</v>
+      </c>
+      <c r="D22" t="s">
+        <v>238</v>
+      </c>
+      <c r="E22" t="s">
+        <v>220</v>
+      </c>
+      <c r="F22" t="s">
+        <v>60</v>
+      </c>
+      <c r="G22" t="s">
+        <v>221</v>
+      </c>
+      <c r="H22" t="s">
+        <v>230</v>
+      </c>
+      <c r="I22">
+        <v>4.2</v>
+      </c>
+      <c r="J22">
+        <v>4.1</v>
+      </c>
+      <c r="K22" t="s">
+        <v>271</v>
+      </c>
+      <c r="L22" t="s">
+        <v>272</v>
+      </c>
+      <c r="M22" t="s">
+        <v>223</v>
+      </c>
+      <c r="N22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O22">
+        <v>8</v>
+      </c>
+      <c r="P22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>416</v>
+      </c>
+      <c r="R22">
+        <v>14</v>
+      </c>
+      <c r="S22" t="s">
+        <v>417</v>
+      </c>
+      <c r="T22" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="U22" t="s">
+        <v>176</v>
+      </c>
+      <c r="V22" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W22" t="s">
+        <v>177</v>
+      </c>
+      <c r="X22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>418</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" t="s">
+        <v>420</v>
+      </c>
+      <c r="D23" t="s">
+        <v>246</v>
+      </c>
+      <c r="E23" t="s">
+        <v>220</v>
+      </c>
+      <c r="F23" t="s">
+        <v>60</v>
+      </c>
+      <c r="G23" t="s">
+        <v>221</v>
+      </c>
+      <c r="H23" t="s">
+        <v>247</v>
+      </c>
+      <c r="I23">
+        <v>6.6</v>
+      </c>
+      <c r="J23">
+        <v>6.5</v>
+      </c>
+      <c r="K23" t="s">
+        <v>271</v>
+      </c>
+      <c r="L23" t="s">
+        <v>272</v>
+      </c>
+      <c r="M23" t="s">
+        <v>223</v>
+      </c>
+      <c r="N23" t="s">
+        <v>38</v>
+      </c>
+      <c r="O23">
+        <v>14</v>
+      </c>
+      <c r="P23" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>421</v>
+      </c>
+      <c r="R23">
+        <v>23</v>
+      </c>
+      <c r="S23" t="s">
+        <v>422</v>
+      </c>
+      <c r="T23" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="U23" t="s">
+        <v>423</v>
+      </c>
+      <c r="V23" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W23" t="s">
+        <v>424</v>
+      </c>
+      <c r="X23" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>425</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" t="s">
+        <v>427</v>
+      </c>
+      <c r="D24" t="s">
+        <v>255</v>
+      </c>
+      <c r="E24" t="s">
+        <v>220</v>
+      </c>
+      <c r="F24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" t="s">
+        <v>230</v>
+      </c>
+      <c r="H24" t="s">
+        <v>247</v>
+      </c>
+      <c r="I24">
+        <v>2.4</v>
+      </c>
+      <c r="J24">
+        <v>2.4</v>
+      </c>
+      <c r="K24" t="s">
+        <v>271</v>
+      </c>
+      <c r="L24" t="s">
+        <v>272</v>
+      </c>
+      <c r="M24" t="s">
+        <v>223</v>
+      </c>
+      <c r="N24" t="s">
+        <v>38</v>
+      </c>
+      <c r="O24">
+        <v>6</v>
+      </c>
+      <c r="P24" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>428</v>
+      </c>
+      <c r="R24">
+        <v>9</v>
+      </c>
+      <c r="S24" t="s">
+        <v>429</v>
+      </c>
+      <c r="T24" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U24" t="s">
+        <v>430</v>
+      </c>
+      <c r="V24" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W24" t="s">
+        <v>431</v>
+      </c>
+      <c r="X24" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>432</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>434</v>
+      </c>
+      <c r="D25" t="s">
+        <v>263</v>
+      </c>
+      <c r="E25" t="s">
+        <v>220</v>
+      </c>
+      <c r="F25" t="s">
+        <v>60</v>
+      </c>
+      <c r="G25" t="s">
+        <v>247</v>
+      </c>
+      <c r="H25" t="s">
+        <v>222</v>
+      </c>
+      <c r="I25">
+        <v>1.7</v>
+      </c>
+      <c r="J25">
+        <v>1.3</v>
+      </c>
+      <c r="K25" t="s">
+        <v>271</v>
+      </c>
+      <c r="L25" t="s">
+        <v>272</v>
+      </c>
+      <c r="M25" t="s">
+        <v>223</v>
+      </c>
+      <c r="N25" t="s">
+        <v>38</v>
+      </c>
+      <c r="O25">
+        <v>3</v>
+      </c>
+      <c r="P25" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>435</v>
+      </c>
+      <c r="R25">
+        <v>3</v>
+      </c>
+      <c r="S25" t="s">
+        <v>436</v>
+      </c>
+      <c r="T25" t="s">
+        <v>113</v>
+      </c>
+      <c r="U25" t="s">
+        <v>114</v>
+      </c>
+      <c r="V25" t="s">
+        <v>115</v>
+      </c>
+      <c r="W25" t="s">
+        <v>116</v>
+      </c>
+      <c r="X25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>437</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>438</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AA1"/>
+  <hyperlinks>
+    <hyperlink ref="X2" r:id="rId1"/>
+    <hyperlink ref="Y2" r:id="rId2"/>
+    <hyperlink ref="X3" r:id="rId3"/>
+    <hyperlink ref="Y3" r:id="rId4"/>
+    <hyperlink ref="X4" r:id="rId5"/>
+    <hyperlink ref="Y4" r:id="rId6"/>
+    <hyperlink ref="X5" r:id="rId7"/>
+    <hyperlink ref="Y5" r:id="rId8"/>
+    <hyperlink ref="X6" r:id="rId9"/>
+    <hyperlink ref="Y6" r:id="rId10"/>
+    <hyperlink ref="X7" r:id="rId11"/>
+    <hyperlink ref="Y7" r:id="rId12"/>
+    <hyperlink ref="X8" r:id="rId13"/>
+    <hyperlink ref="Y8" r:id="rId14"/>
+    <hyperlink ref="X9" r:id="rId15"/>
+    <hyperlink ref="Y9" r:id="rId16"/>
+    <hyperlink ref="X10" r:id="rId17"/>
+    <hyperlink ref="Y10" r:id="rId18"/>
+    <hyperlink ref="X11" r:id="rId19"/>
+    <hyperlink ref="Y11" r:id="rId20"/>
+    <hyperlink ref="X12" r:id="rId21"/>
+    <hyperlink ref="Y12" r:id="rId22"/>
+    <hyperlink ref="X13" r:id="rId23"/>
+    <hyperlink ref="Y13" r:id="rId24"/>
+    <hyperlink ref="X14" r:id="rId25"/>
+    <hyperlink ref="Y14" r:id="rId26"/>
+    <hyperlink ref="X15" r:id="rId27"/>
+    <hyperlink ref="Y15" r:id="rId28"/>
+    <hyperlink ref="X16" r:id="rId29"/>
+    <hyperlink ref="Y16" r:id="rId30"/>
+    <hyperlink ref="X17" r:id="rId31"/>
+    <hyperlink ref="Y17" r:id="rId32"/>
+    <hyperlink ref="X18" r:id="rId33"/>
+    <hyperlink ref="Y18" r:id="rId34"/>
+    <hyperlink ref="X19" r:id="rId35"/>
+    <hyperlink ref="Y19" r:id="rId36"/>
+    <hyperlink ref="X20" r:id="rId37"/>
+    <hyperlink ref="Y20" r:id="rId38"/>
+    <hyperlink ref="X21" r:id="rId39"/>
+    <hyperlink ref="Y21" r:id="rId40"/>
+    <hyperlink ref="X22" r:id="rId41"/>
+    <hyperlink ref="Y22" r:id="rId42"/>
+    <hyperlink ref="X23" r:id="rId43"/>
+    <hyperlink ref="Y23" r:id="rId44"/>
+    <hyperlink ref="X24" r:id="rId45"/>
+    <hyperlink ref="Y24" r:id="rId46"/>
+    <hyperlink ref="X25" r:id="rId47"/>
+    <hyperlink ref="Y25" r:id="rId48"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:X25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:24" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>3</v>
       </c>
@@ -3415,34 +6087,61 @@
         <v>9</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>270</v>
+        <v>439</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>271</v>
+        <v>440</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>272</v>
+        <v>441</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>273</v>
+        <v>442</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>274</v>
+        <v>443</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>275</v>
+        <v>444</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>276</v>
+        <v>445</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>277</v>
+        <v>446</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>278</v>
+        <v>447</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="R1" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="S1" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>452</v>
+      </c>
+      <c r="U1" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="V1" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="W1" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="X1" s="4" t="s">
+        <v>456</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -3488,8 +6187,35 @@
       <c r="O2" t="s">
         <v>44</v>
       </c>
+      <c r="P2" t="s">
+        <v>270</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>37</v>
+      </c>
+      <c r="R2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S2">
+        <v>28</v>
+      </c>
+      <c r="T2" t="s">
+        <v>39</v>
+      </c>
+      <c r="U2" t="s">
+        <v>273</v>
+      </c>
+      <c r="V2">
+        <v>51</v>
+      </c>
+      <c r="W2" t="s">
+        <v>39</v>
+      </c>
+      <c r="X2" t="s">
+        <v>277</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -3535,8 +6261,35 @@
       <c r="O3" t="s">
         <v>55</v>
       </c>
+      <c r="P3" t="s">
+        <v>280</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>37</v>
+      </c>
+      <c r="R3" t="s">
+        <v>38</v>
+      </c>
+      <c r="S3">
+        <v>28</v>
+      </c>
+      <c r="T3" t="s">
+        <v>39</v>
+      </c>
+      <c r="U3" t="s">
+        <v>281</v>
+      </c>
+      <c r="V3">
+        <v>59</v>
+      </c>
+      <c r="W3" t="s">
+        <v>39</v>
+      </c>
+      <c r="X3" t="s">
+        <v>285</v>
+      </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -3582,8 +6335,35 @@
       <c r="O4" t="s">
         <v>67</v>
       </c>
+      <c r="P4" t="s">
+        <v>288</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>37</v>
+      </c>
+      <c r="R4" t="s">
+        <v>38</v>
+      </c>
+      <c r="S4">
+        <v>7</v>
+      </c>
+      <c r="T4" t="s">
+        <v>39</v>
+      </c>
+      <c r="U4" t="s">
+        <v>289</v>
+      </c>
+      <c r="V4">
+        <v>17</v>
+      </c>
+      <c r="W4" t="s">
+        <v>39</v>
+      </c>
+      <c r="X4" t="s">
+        <v>293</v>
+      </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -3629,8 +6409,35 @@
       <c r="O5" t="s">
         <v>76</v>
       </c>
+      <c r="P5" t="s">
+        <v>296</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>37</v>
+      </c>
+      <c r="R5" t="s">
+        <v>38</v>
+      </c>
+      <c r="S5">
+        <v>11</v>
+      </c>
+      <c r="T5" t="s">
+        <v>39</v>
+      </c>
+      <c r="U5" t="s">
+        <v>297</v>
+      </c>
+      <c r="V5">
+        <v>23</v>
+      </c>
+      <c r="W5" t="s">
+        <v>39</v>
+      </c>
+      <c r="X5" t="s">
+        <v>300</v>
+      </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>80</v>
       </c>
@@ -3676,8 +6483,35 @@
       <c r="O6" t="s">
         <v>86</v>
       </c>
+      <c r="P6" t="s">
+        <v>303</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>37</v>
+      </c>
+      <c r="R6" t="s">
+        <v>38</v>
+      </c>
+      <c r="S6">
+        <v>11</v>
+      </c>
+      <c r="T6" t="s">
+        <v>39</v>
+      </c>
+      <c r="U6" t="s">
+        <v>304</v>
+      </c>
+      <c r="V6">
+        <v>20</v>
+      </c>
+      <c r="W6" t="s">
+        <v>39</v>
+      </c>
+      <c r="X6" t="s">
+        <v>306</v>
+      </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>90</v>
       </c>
@@ -3723,8 +6557,35 @@
       <c r="O7" t="s">
         <v>95</v>
       </c>
+      <c r="P7" t="s">
+        <v>309</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>37</v>
+      </c>
+      <c r="R7" t="s">
+        <v>38</v>
+      </c>
+      <c r="S7">
+        <v>12</v>
+      </c>
+      <c r="T7" t="s">
+        <v>39</v>
+      </c>
+      <c r="U7" t="s">
+        <v>310</v>
+      </c>
+      <c r="V7">
+        <v>30</v>
+      </c>
+      <c r="W7" t="s">
+        <v>39</v>
+      </c>
+      <c r="X7" t="s">
+        <v>314</v>
+      </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>99</v>
       </c>
@@ -3770,8 +6631,35 @@
       <c r="O8" t="s">
         <v>105</v>
       </c>
+      <c r="P8" t="s">
+        <v>317</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>37</v>
+      </c>
+      <c r="R8" t="s">
+        <v>38</v>
+      </c>
+      <c r="S8">
+        <v>17</v>
+      </c>
+      <c r="T8" t="s">
+        <v>39</v>
+      </c>
+      <c r="U8" t="s">
+        <v>318</v>
+      </c>
+      <c r="V8">
+        <v>31</v>
+      </c>
+      <c r="W8" t="s">
+        <v>39</v>
+      </c>
+      <c r="X8" t="s">
+        <v>321</v>
+      </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>109</v>
       </c>
@@ -3817,8 +6705,35 @@
       <c r="O9" t="s">
         <v>116</v>
       </c>
+      <c r="P9" t="s">
+        <v>324</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>37</v>
+      </c>
+      <c r="R9" t="s">
+        <v>38</v>
+      </c>
+      <c r="S9">
+        <v>15</v>
+      </c>
+      <c r="T9" t="s">
+        <v>39</v>
+      </c>
+      <c r="U9" t="s">
+        <v>325</v>
+      </c>
+      <c r="V9">
+        <v>27</v>
+      </c>
+      <c r="W9" t="s">
+        <v>39</v>
+      </c>
+      <c r="X9" t="s">
+        <v>328</v>
+      </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>120</v>
       </c>
@@ -3864,8 +6779,35 @@
       <c r="O10" t="s">
         <v>125</v>
       </c>
+      <c r="P10" t="s">
+        <v>331</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>37</v>
+      </c>
+      <c r="R10" t="s">
+        <v>38</v>
+      </c>
+      <c r="S10">
+        <v>16</v>
+      </c>
+      <c r="T10" t="s">
+        <v>39</v>
+      </c>
+      <c r="U10" t="s">
+        <v>332</v>
+      </c>
+      <c r="V10">
+        <v>38</v>
+      </c>
+      <c r="W10" t="s">
+        <v>39</v>
+      </c>
+      <c r="X10" t="s">
+        <v>336</v>
+      </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>129</v>
       </c>
@@ -3911,8 +6853,35 @@
       <c r="O11" t="s">
         <v>139</v>
       </c>
+      <c r="P11" t="s">
+        <v>339</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>133</v>
+      </c>
+      <c r="R11" t="s">
+        <v>38</v>
+      </c>
+      <c r="S11">
+        <v>30</v>
+      </c>
+      <c r="T11" t="s">
+        <v>39</v>
+      </c>
+      <c r="U11" t="s">
+        <v>340</v>
+      </c>
+      <c r="V11">
+        <v>51</v>
+      </c>
+      <c r="W11" t="s">
+        <v>39</v>
+      </c>
+      <c r="X11" t="s">
+        <v>344</v>
+      </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>143</v>
       </c>
@@ -3958,8 +6927,35 @@
       <c r="O12" t="s">
         <v>149</v>
       </c>
+      <c r="P12" t="s">
+        <v>347</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>133</v>
+      </c>
+      <c r="R12" t="s">
+        <v>38</v>
+      </c>
+      <c r="S12">
+        <v>21</v>
+      </c>
+      <c r="T12" t="s">
+        <v>39</v>
+      </c>
+      <c r="U12" t="s">
+        <v>348</v>
+      </c>
+      <c r="V12">
+        <v>35</v>
+      </c>
+      <c r="W12" t="s">
+        <v>39</v>
+      </c>
+      <c r="X12" t="s">
+        <v>95</v>
+      </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>153</v>
       </c>
@@ -4005,8 +7001,35 @@
       <c r="O13" t="s">
         <v>158</v>
       </c>
+      <c r="P13" t="s">
+        <v>352</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>133</v>
+      </c>
+      <c r="R13" t="s">
+        <v>38</v>
+      </c>
+      <c r="S13">
+        <v>9</v>
+      </c>
+      <c r="T13" t="s">
+        <v>39</v>
+      </c>
+      <c r="U13" t="s">
+        <v>353</v>
+      </c>
+      <c r="V13">
+        <v>33</v>
+      </c>
+      <c r="W13" t="s">
+        <v>39</v>
+      </c>
+      <c r="X13" t="s">
+        <v>357</v>
+      </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>162</v>
       </c>
@@ -4052,8 +7075,35 @@
       <c r="O14" t="s">
         <v>168</v>
       </c>
+      <c r="P14" t="s">
+        <v>360</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>133</v>
+      </c>
+      <c r="R14" t="s">
+        <v>38</v>
+      </c>
+      <c r="S14">
+        <v>18</v>
+      </c>
+      <c r="T14" t="s">
+        <v>39</v>
+      </c>
+      <c r="U14" t="s">
+        <v>361</v>
+      </c>
+      <c r="V14">
+        <v>22</v>
+      </c>
+      <c r="W14" t="s">
+        <v>39</v>
+      </c>
+      <c r="X14" t="s">
+        <v>364</v>
+      </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>172</v>
       </c>
@@ -4099,8 +7149,35 @@
       <c r="O15" t="s">
         <v>177</v>
       </c>
+      <c r="P15" t="s">
+        <v>367</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>133</v>
+      </c>
+      <c r="R15" t="s">
+        <v>38</v>
+      </c>
+      <c r="S15">
+        <v>12</v>
+      </c>
+      <c r="T15" t="s">
+        <v>39</v>
+      </c>
+      <c r="U15" t="s">
+        <v>368</v>
+      </c>
+      <c r="V15">
+        <v>34</v>
+      </c>
+      <c r="W15" t="s">
+        <v>39</v>
+      </c>
+      <c r="X15" t="s">
+        <v>371</v>
+      </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>181</v>
       </c>
@@ -4146,8 +7223,35 @@
       <c r="O16" t="s">
         <v>186</v>
       </c>
+      <c r="P16" t="s">
+        <v>374</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>133</v>
+      </c>
+      <c r="R16" t="s">
+        <v>38</v>
+      </c>
+      <c r="S16">
+        <v>25</v>
+      </c>
+      <c r="T16" t="s">
+        <v>39</v>
+      </c>
+      <c r="U16" t="s">
+        <v>375</v>
+      </c>
+      <c r="V16">
+        <v>46</v>
+      </c>
+      <c r="W16" t="s">
+        <v>39</v>
+      </c>
+      <c r="X16" t="s">
+        <v>378</v>
+      </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>190</v>
       </c>
@@ -4193,8 +7297,35 @@
       <c r="O17" t="s">
         <v>198</v>
       </c>
+      <c r="P17" t="s">
+        <v>381</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>193</v>
+      </c>
+      <c r="R17" t="s">
+        <v>38</v>
+      </c>
+      <c r="S17">
+        <v>23</v>
+      </c>
+      <c r="T17" t="s">
+        <v>39</v>
+      </c>
+      <c r="U17" t="s">
+        <v>382</v>
+      </c>
+      <c r="V17">
+        <v>30</v>
+      </c>
+      <c r="W17" t="s">
+        <v>39</v>
+      </c>
+      <c r="X17" t="s">
+        <v>386</v>
+      </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>202</v>
       </c>
@@ -4240,8 +7371,35 @@
       <c r="O18" t="s">
         <v>168</v>
       </c>
+      <c r="P18" t="s">
+        <v>389</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>193</v>
+      </c>
+      <c r="R18" t="s">
+        <v>38</v>
+      </c>
+      <c r="S18">
+        <v>12</v>
+      </c>
+      <c r="T18" t="s">
+        <v>39</v>
+      </c>
+      <c r="U18" t="s">
+        <v>390</v>
+      </c>
+      <c r="V18">
+        <v>14</v>
+      </c>
+      <c r="W18" t="s">
+        <v>39</v>
+      </c>
+      <c r="X18" t="s">
+        <v>259</v>
+      </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>210</v>
       </c>
@@ -4287,8 +7445,35 @@
       <c r="O19" t="s">
         <v>215</v>
       </c>
+      <c r="P19" t="s">
+        <v>394</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>193</v>
+      </c>
+      <c r="R19" t="s">
+        <v>38</v>
+      </c>
+      <c r="S19">
+        <v>19</v>
+      </c>
+      <c r="T19" t="s">
+        <v>39</v>
+      </c>
+      <c r="U19" t="s">
+        <v>395</v>
+      </c>
+      <c r="V19">
+        <v>28</v>
+      </c>
+      <c r="W19" t="s">
+        <v>39</v>
+      </c>
+      <c r="X19" t="s">
+        <v>398</v>
+      </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>219</v>
       </c>
@@ -4334,8 +7519,35 @@
       <c r="O20" t="s">
         <v>105</v>
       </c>
+      <c r="P20" t="s">
+        <v>401</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>223</v>
+      </c>
+      <c r="R20" t="s">
+        <v>38</v>
+      </c>
+      <c r="S20">
+        <v>17</v>
+      </c>
+      <c r="T20" t="s">
+        <v>39</v>
+      </c>
+      <c r="U20" t="s">
+        <v>402</v>
+      </c>
+      <c r="V20">
+        <v>27</v>
+      </c>
+      <c r="W20" t="s">
+        <v>39</v>
+      </c>
+      <c r="X20" t="s">
+        <v>405</v>
+      </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>229</v>
       </c>
@@ -4381,8 +7593,35 @@
       <c r="O21" t="s">
         <v>234</v>
       </c>
+      <c r="P21" t="s">
+        <v>408</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>223</v>
+      </c>
+      <c r="R21" t="s">
+        <v>38</v>
+      </c>
+      <c r="S21">
+        <v>9</v>
+      </c>
+      <c r="T21" t="s">
+        <v>39</v>
+      </c>
+      <c r="U21" t="s">
+        <v>409</v>
+      </c>
+      <c r="V21">
+        <v>13</v>
+      </c>
+      <c r="W21" t="s">
+        <v>39</v>
+      </c>
+      <c r="X21" t="s">
+        <v>412</v>
+      </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>238</v>
       </c>
@@ -4428,8 +7667,35 @@
       <c r="O22" t="s">
         <v>242</v>
       </c>
+      <c r="P22" t="s">
+        <v>415</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>223</v>
+      </c>
+      <c r="R22" t="s">
+        <v>38</v>
+      </c>
+      <c r="S22">
+        <v>8</v>
+      </c>
+      <c r="T22" t="s">
+        <v>39</v>
+      </c>
+      <c r="U22" t="s">
+        <v>416</v>
+      </c>
+      <c r="V22">
+        <v>14</v>
+      </c>
+      <c r="W22" t="s">
+        <v>39</v>
+      </c>
+      <c r="X22" t="s">
+        <v>177</v>
+      </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>246</v>
       </c>
@@ -4475,8 +7741,35 @@
       <c r="O23" t="s">
         <v>251</v>
       </c>
+      <c r="P23" t="s">
+        <v>420</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>223</v>
+      </c>
+      <c r="R23" t="s">
+        <v>38</v>
+      </c>
+      <c r="S23">
+        <v>14</v>
+      </c>
+      <c r="T23" t="s">
+        <v>39</v>
+      </c>
+      <c r="U23" t="s">
+        <v>421</v>
+      </c>
+      <c r="V23">
+        <v>23</v>
+      </c>
+      <c r="W23" t="s">
+        <v>39</v>
+      </c>
+      <c r="X23" t="s">
+        <v>424</v>
+      </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>255</v>
       </c>
@@ -4522,8 +7815,35 @@
       <c r="O24" t="s">
         <v>259</v>
       </c>
+      <c r="P24" t="s">
+        <v>427</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>223</v>
+      </c>
+      <c r="R24" t="s">
+        <v>38</v>
+      </c>
+      <c r="S24">
+        <v>6</v>
+      </c>
+      <c r="T24" t="s">
+        <v>39</v>
+      </c>
+      <c r="U24" t="s">
+        <v>428</v>
+      </c>
+      <c r="V24">
+        <v>9</v>
+      </c>
+      <c r="W24" t="s">
+        <v>39</v>
+      </c>
+      <c r="X24" t="s">
+        <v>431</v>
+      </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>263</v>
       </c>
@@ -4569,9 +7889,36 @@
       <c r="O25" t="s">
         <v>267</v>
       </c>
+      <c r="P25" t="s">
+        <v>434</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>223</v>
+      </c>
+      <c r="R25" t="s">
+        <v>38</v>
+      </c>
+      <c r="S25">
+        <v>3</v>
+      </c>
+      <c r="T25" t="s">
+        <v>39</v>
+      </c>
+      <c r="U25" t="s">
+        <v>435</v>
+      </c>
+      <c r="V25">
+        <v>3</v>
+      </c>
+      <c r="W25" t="s">
+        <v>115</v>
+      </c>
+      <c r="X25" t="s">
+        <v>116</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O1"/>
+  <autoFilter ref="A1:X1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Auto-collect traffic data: 2026-09-29 01:11 PM IST
</commit_message>
<xml_diff>
--- a/output/excel/Metro_vs_Car_Data_2026-09-29_Tue.xlsx
+++ b/output/excel/Metro_vs_Car_Data_2026-09-29_Tue.xlsx
@@ -6,14 +6,15 @@
   <sheets>
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="10_00 AM" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="All Periods Combined" state="visible" r:id="rId6"/>
+    <sheet sheetId="3" name="1_00 PM" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="All Periods Combined" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1614" uniqueCount="457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2370" uniqueCount="640">
   <si>
     <t>Date</t>
   </si>
@@ -1332,6 +1333,525 @@
     <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/10_00_AM/MC-24/car.jpg</t>
   </si>
   <si>
+    <t>9/29/2026, 1:02:53 PM</t>
+  </si>
+  <si>
+    <t>1:00 PM</t>
+  </si>
+  <si>
+    <t>Tuesday (Weekday) - Mid-day Off-Peak</t>
+  </si>
+  <si>
+    <t> | 31 min | 6:00 AM—6:31 AM | Blue Line | 6:00 AM from Dakshineswar | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 58 min | 12.2 km | via Barrackpore Trunk Rd | Fastest route, despite slowdown on SH 1 causing 7-min delay | Details | Preview</t>
+  </si>
+  <si>
+    <t>27 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>1.87x</t>
+  </si>
+  <si>
+    <t>46.6% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-01/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-01/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:03:11 PM</t>
+  </si>
+  <si>
+    <t> | 30 min | 6:00 AM—6:30 AM | Blue Line | 6:00 AM from Shahid Khudiram | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 1 hr 5 min | 15.5 km | via Netaji Subhas Chandra Bose Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>35 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.17x</t>
+  </si>
+  <si>
+    <t>53.8% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-02/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-02/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:03:28 PM</t>
+  </si>
+  <si>
+    <t> | 54 min | 3.8 km | via Belgachia Rd/Khudiram Bose Sarani</t>
+  </si>
+  <si>
+    <t> | 18 min | 3.5 km | via Belgachia Rd/Khudiram Bose Sarani | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>36 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.33x</t>
+  </si>
+  <si>
+    <t>66.7% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-03/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-03/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:04:00 PM</t>
+  </si>
+  <si>
+    <t> | 11 min | 12:36 PM—12:47 PM | Blue Line | 12:36 PM from Shyambazar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 39 min | 6.2 km | via Jatindra Mohan Ave | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>28 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>3.55x</t>
+  </si>
+  <si>
+    <t>71.8% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-04/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-04/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:04:32 PM</t>
+  </si>
+  <si>
+    <t> | 11 min | 12:36 PM—12:47 PM | Blue Line | 12:36 PM from Kalighat | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 24 min | 5.1 km | via Shyama Prasad Mukherjee Rd and Ashutosh Mukherjee Rd | Fastest route, despite heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>13 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.18x</t>
+  </si>
+  <si>
+    <t>54.2% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-05/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-05/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:04:49 PM</t>
+  </si>
+  <si>
+    <t> | 15 min | 6:00 AM—6:15 AM | Blue Line | 6:00 AM from Dakshineswar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 28 min | 7.0 km | via Barrackpore Trunk Rd | Fastest route, despite slowdown on SH 1 causing 9-min delay | Details | Preview</t>
+  </si>
+  <si>
+    <t>46.4% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-06/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-06/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:05:07 PM</t>
+  </si>
+  <si>
+    <t> | 23 min | 6:31 AM—6:54 AM | Blue Line</t>
+  </si>
+  <si>
+    <t> | 31 min | 8.1 km | via Chowringee Rd/Jawaharlal Nehru Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.35x</t>
+  </si>
+  <si>
+    <t>25.8% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-07/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-07/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:05:24 PM</t>
+  </si>
+  <si>
+    <t> | 17 min | 6:10 AM—6:27 AM | Blue Line | 6:10 AM from Mahanayak Uttam Kumar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 26 min | 6.4 km | via Netaji Subhas Chandra Bose Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.53x</t>
+  </si>
+  <si>
+    <t>34.6% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-08/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-08/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:05:42 PM</t>
+  </si>
+  <si>
+    <t> | 16 min | 6:15 AM—6:31 AM | Blue Line</t>
+  </si>
+  <si>
+    <t> | 49 min | 8.6 km | via Jessore Rd and Lock Gate Rd | Fastest route, despite much heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>33 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>3.06x</t>
+  </si>
+  <si>
+    <t>67.3% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-09/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-09/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:06:01 PM</t>
+  </si>
+  <si>
+    <t> | 30 min | 6:02 AM—6:32 AM | Green Line</t>
+  </si>
+  <si>
+    <t> | 58 min | 12.3 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.93x</t>
+  </si>
+  <si>
+    <t>48.3% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-10/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-10/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:06:32 PM</t>
+  </si>
+  <si>
+    <t> | 21 min | 12:31 PM—12:52 PM | Green Line | 12:31 PM from Sealdah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 32 min | 8.0 km | via Beleghata Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.52x</t>
+  </si>
+  <si>
+    <t>34.4% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-11/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-11/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:06:50 PM</t>
+  </si>
+  <si>
+    <t> | 9 min | 6:02 AM—6:11 AM | Green Line</t>
+  </si>
+  <si>
+    <t> | 50 min | 7.2 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>41 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>5.56x</t>
+  </si>
+  <si>
+    <t>82.0% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-12/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-12/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:07:24 PM</t>
+  </si>
+  <si>
+    <t> | 18 min | 12:34 PM—12:52 PM | Green Line | 12:34 PM from Phoolbagan | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 18 min | 4.9 km | via Narkeldanga Main Rd | Fastest route, the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-13/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-13/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:07:42 PM</t>
+  </si>
+  <si>
+    <t> | 12 min | 6:02 AM—6:14 AM | Green Line</t>
+  </si>
+  <si>
+    <t> | 45 min | 7.6 km | via Kali Krishna Tagore St | Fastest route, despite much heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>3.75x</t>
+  </si>
+  <si>
+    <t>73.3% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-14/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-14/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:08:13 PM</t>
+  </si>
+  <si>
+    <t> | 25 min | 12:37 PM—1:02 PM | Green Line | 12:37 PM from Esplanade | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t> | 35 min | 13.3 km | via Indira Gandhi Sarani and Park St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.40x</t>
+  </si>
+  <si>
+    <t>28.6% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-15/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-15/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:08:30 PM</t>
+  </si>
+  <si>
+    <t> | 28 min | 7:40 AM—8:08 AM | Orange Line | 7:40 AM from Kavi Subhash | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 24 min | 9.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route, the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>0.86x</t>
+  </si>
+  <si>
+    <t>14.3% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-16/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-16/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:09:01 PM</t>
+  </si>
+  <si>
+    <t> | 12 min | 12:36 PM—12:48 PM | Orange Line | 12:36 PM from Hemanta Mukhopadhyay | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t> | 10 min | 4.4 km | via Bangaon - Kulpi Rd/Biswa Bangla Sarani/Eastern Metropolitan Bypass/Thakurnagar - Panchpota Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>0.83x</t>
+  </si>
+  <si>
+    <t>16.7% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-17/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-17/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:09:19 PM</t>
+  </si>
+  <si>
+    <t> | 23 min | 7:40 AM—8:03 AM | Orange Line | 7:40 AM from Kavi Subhash | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 22 min | 8.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route, the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>0.96x</t>
+  </si>
+  <si>
+    <t>4.3% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-18/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-18/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:09:37 PM</t>
+  </si>
+  <si>
+    <t> | 17 min | 6:40 AM—6:57 AM | Purple Line | 6:40 AM from Joka | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 26 min | 7.8 km | via NH 12 | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-19/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-19/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:09:53 PM</t>
+  </si>
+  <si>
+    <t> | 51 min | 3.7 km | via NH 12</t>
+  </si>
+  <si>
+    <t> | 13 min | 3.7 km | via NH 12 | Fastest route, despite slowdown on NH 12 causing 5-min delay | Details | Preview</t>
+  </si>
+  <si>
+    <t>38 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.25x</t>
+  </si>
+  <si>
+    <t>74.5% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-20/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-20/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:10:09 PM</t>
+  </si>
+  <si>
+    <t> | 57 min | 4.1 km | via NH 12 | Details | Preview</t>
+  </si>
+  <si>
+    <t> | 13 min | 4.1 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>44 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.23x</t>
+  </si>
+  <si>
+    <t>77.2% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-21/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-21/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:10:26 PM</t>
+  </si>
+  <si>
+    <t> | 14 min | 6:40 AM—6:54 AM | Purple Line | 6:40 AM from Joka | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-22/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-22/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:10:43 PM</t>
+  </si>
+  <si>
+    <t> | 33 min | 2.4 km | via NH 12 | Details | Preview</t>
+  </si>
+  <si>
+    <t> | 10 min | 2.4 km | via NH 12 | Fastest route, despite slowdown on NH 12 causing 5-min delay | Details | Preview</t>
+  </si>
+  <si>
+    <t>23 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.30x</t>
+  </si>
+  <si>
+    <t>69.7% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-23/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-23/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 1:11:01 PM</t>
+  </si>
+  <si>
+    <t> | 18 min | 1.3 km | via NH 12 | Details | Preview</t>
+  </si>
+  <si>
+    <t> | 3 min | 1.3 km | via NH 12 | Fastest route, the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>15 min (Car Faster)</t>
+  </si>
+  <si>
+    <t>0.17x</t>
+  </si>
+  <si>
+    <t>83.3% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-24/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-24/car.jpg</t>
+  </si>
+  <si>
     <t>12:00 AM Scraped At</t>
   </si>
   <si>
@@ -1384,6 +1904,36 @@
   </si>
   <si>
     <t>10:00 AM Savings (%)</t>
+  </si>
+  <si>
+    <t>1:00 PM Scraped At</t>
+  </si>
+  <si>
+    <t>1:00 PM Actual Metro</t>
+  </si>
+  <si>
+    <t>1:00 PM Metro Walk</t>
+  </si>
+  <si>
+    <t>1:00 PM Metro (min)</t>
+  </si>
+  <si>
+    <t>1:00 PM Metro Route</t>
+  </si>
+  <si>
+    <t>1:00 PM Metro Raw Details</t>
+  </si>
+  <si>
+    <t>1:00 PM Car (min)</t>
+  </si>
+  <si>
+    <t>1:00 PM Faster Mode</t>
+  </si>
+  <si>
+    <t>1:00 PM Savings (%)</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -6064,10 +6614,2147 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X25"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:24" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>439</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2">
+        <v>15</v>
+      </c>
+      <c r="J2">
+        <v>12.2</v>
+      </c>
+      <c r="K2" t="s">
+        <v>440</v>
+      </c>
+      <c r="L2" t="s">
+        <v>441</v>
+      </c>
+      <c r="M2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2">
+        <v>31</v>
+      </c>
+      <c r="P2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>442</v>
+      </c>
+      <c r="R2">
+        <v>58</v>
+      </c>
+      <c r="S2" t="s">
+        <v>443</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="U2" t="s">
+        <v>445</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W2" t="s">
+        <v>446</v>
+      </c>
+      <c r="X2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>447</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>449</v>
+      </c>
+      <c r="D3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3">
+        <v>14.9</v>
+      </c>
+      <c r="J3">
+        <v>15.5</v>
+      </c>
+      <c r="K3" t="s">
+        <v>440</v>
+      </c>
+      <c r="L3" t="s">
+        <v>441</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3">
+        <v>30</v>
+      </c>
+      <c r="P3" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>450</v>
+      </c>
+      <c r="R3">
+        <v>65</v>
+      </c>
+      <c r="S3" t="s">
+        <v>451</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="U3" t="s">
+        <v>453</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W3" t="s">
+        <v>454</v>
+      </c>
+      <c r="X3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>455</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>457</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I4">
+        <v>3.8</v>
+      </c>
+      <c r="J4">
+        <v>3.5</v>
+      </c>
+      <c r="K4" t="s">
+        <v>440</v>
+      </c>
+      <c r="L4" t="s">
+        <v>441</v>
+      </c>
+      <c r="M4" t="s">
+        <v>38</v>
+      </c>
+      <c r="N4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4">
+        <v>54</v>
+      </c>
+      <c r="P4" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>458</v>
+      </c>
+      <c r="R4">
+        <v>18</v>
+      </c>
+      <c r="S4" t="s">
+        <v>459</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="U4" t="s">
+        <v>461</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="W4" t="s">
+        <v>462</v>
+      </c>
+      <c r="X4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>463</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>465</v>
+      </c>
+      <c r="D5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5">
+        <v>5.1</v>
+      </c>
+      <c r="J5">
+        <v>6.2</v>
+      </c>
+      <c r="K5" t="s">
+        <v>440</v>
+      </c>
+      <c r="L5" t="s">
+        <v>441</v>
+      </c>
+      <c r="M5" t="s">
+        <v>37</v>
+      </c>
+      <c r="N5" t="s">
+        <v>38</v>
+      </c>
+      <c r="O5">
+        <v>11</v>
+      </c>
+      <c r="P5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>466</v>
+      </c>
+      <c r="R5">
+        <v>39</v>
+      </c>
+      <c r="S5" t="s">
+        <v>467</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="U5" t="s">
+        <v>469</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W5" t="s">
+        <v>470</v>
+      </c>
+      <c r="X5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>471</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>473</v>
+      </c>
+      <c r="D6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6">
+        <v>5.2</v>
+      </c>
+      <c r="J6">
+        <v>5.1</v>
+      </c>
+      <c r="K6" t="s">
+        <v>440</v>
+      </c>
+      <c r="L6" t="s">
+        <v>441</v>
+      </c>
+      <c r="M6" t="s">
+        <v>37</v>
+      </c>
+      <c r="N6" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6">
+        <v>11</v>
+      </c>
+      <c r="P6" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>474</v>
+      </c>
+      <c r="R6">
+        <v>24</v>
+      </c>
+      <c r="S6" t="s">
+        <v>475</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="U6" t="s">
+        <v>477</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W6" t="s">
+        <v>478</v>
+      </c>
+      <c r="X6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>479</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>481</v>
+      </c>
+      <c r="D7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I7">
+        <v>6.2</v>
+      </c>
+      <c r="J7">
+        <v>7</v>
+      </c>
+      <c r="K7" t="s">
+        <v>440</v>
+      </c>
+      <c r="L7" t="s">
+        <v>441</v>
+      </c>
+      <c r="M7" t="s">
+        <v>37</v>
+      </c>
+      <c r="N7" t="s">
+        <v>38</v>
+      </c>
+      <c r="O7">
+        <v>15</v>
+      </c>
+      <c r="P7" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>482</v>
+      </c>
+      <c r="R7">
+        <v>28</v>
+      </c>
+      <c r="S7" t="s">
+        <v>483</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="U7" t="s">
+        <v>445</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W7" t="s">
+        <v>484</v>
+      </c>
+      <c r="X7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>485</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>487</v>
+      </c>
+      <c r="D8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" t="s">
+        <v>100</v>
+      </c>
+      <c r="I8">
+        <v>7.8</v>
+      </c>
+      <c r="J8">
+        <v>8.1</v>
+      </c>
+      <c r="K8" t="s">
+        <v>440</v>
+      </c>
+      <c r="L8" t="s">
+        <v>441</v>
+      </c>
+      <c r="M8" t="s">
+        <v>37</v>
+      </c>
+      <c r="N8" t="s">
+        <v>38</v>
+      </c>
+      <c r="O8">
+        <v>23</v>
+      </c>
+      <c r="P8" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>488</v>
+      </c>
+      <c r="R8">
+        <v>31</v>
+      </c>
+      <c r="S8" t="s">
+        <v>489</v>
+      </c>
+      <c r="T8" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="U8" t="s">
+        <v>490</v>
+      </c>
+      <c r="V8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W8" t="s">
+        <v>491</v>
+      </c>
+      <c r="X8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>492</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>494</v>
+      </c>
+      <c r="D9" t="s">
+        <v>109</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" t="s">
+        <v>100</v>
+      </c>
+      <c r="H9" t="s">
+        <v>110</v>
+      </c>
+      <c r="I9">
+        <v>7.1</v>
+      </c>
+      <c r="J9">
+        <v>6.4</v>
+      </c>
+      <c r="K9" t="s">
+        <v>440</v>
+      </c>
+      <c r="L9" t="s">
+        <v>441</v>
+      </c>
+      <c r="M9" t="s">
+        <v>37</v>
+      </c>
+      <c r="N9" t="s">
+        <v>38</v>
+      </c>
+      <c r="O9">
+        <v>17</v>
+      </c>
+      <c r="P9" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>495</v>
+      </c>
+      <c r="R9">
+        <v>26</v>
+      </c>
+      <c r="S9" t="s">
+        <v>496</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="U9" t="s">
+        <v>497</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W9" t="s">
+        <v>498</v>
+      </c>
+      <c r="X9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>499</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>501</v>
+      </c>
+      <c r="D10" t="s">
+        <v>120</v>
+      </c>
+      <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10">
+        <v>8.8</v>
+      </c>
+      <c r="J10">
+        <v>8.6</v>
+      </c>
+      <c r="K10" t="s">
+        <v>440</v>
+      </c>
+      <c r="L10" t="s">
+        <v>441</v>
+      </c>
+      <c r="M10" t="s">
+        <v>37</v>
+      </c>
+      <c r="N10" t="s">
+        <v>38</v>
+      </c>
+      <c r="O10">
+        <v>16</v>
+      </c>
+      <c r="P10" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>502</v>
+      </c>
+      <c r="R10">
+        <v>49</v>
+      </c>
+      <c r="S10" t="s">
+        <v>503</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="U10" t="s">
+        <v>505</v>
+      </c>
+      <c r="V10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W10" t="s">
+        <v>506</v>
+      </c>
+      <c r="X10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>507</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>509</v>
+      </c>
+      <c r="D11" t="s">
+        <v>129</v>
+      </c>
+      <c r="E11" t="s">
+        <v>130</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>131</v>
+      </c>
+      <c r="H11" t="s">
+        <v>132</v>
+      </c>
+      <c r="I11">
+        <v>14.2</v>
+      </c>
+      <c r="J11">
+        <v>12.3</v>
+      </c>
+      <c r="K11" t="s">
+        <v>440</v>
+      </c>
+      <c r="L11" t="s">
+        <v>441</v>
+      </c>
+      <c r="M11" t="s">
+        <v>133</v>
+      </c>
+      <c r="N11" t="s">
+        <v>38</v>
+      </c>
+      <c r="O11">
+        <v>30</v>
+      </c>
+      <c r="P11" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>510</v>
+      </c>
+      <c r="R11">
+        <v>58</v>
+      </c>
+      <c r="S11" t="s">
+        <v>511</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>468</v>
+      </c>
+      <c r="U11" t="s">
+        <v>512</v>
+      </c>
+      <c r="V11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W11" t="s">
+        <v>513</v>
+      </c>
+      <c r="X11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>514</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>516</v>
+      </c>
+      <c r="D12" t="s">
+        <v>143</v>
+      </c>
+      <c r="E12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" t="s">
+        <v>144</v>
+      </c>
+      <c r="H12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I12">
+        <v>8.6</v>
+      </c>
+      <c r="J12">
+        <v>8</v>
+      </c>
+      <c r="K12" t="s">
+        <v>440</v>
+      </c>
+      <c r="L12" t="s">
+        <v>441</v>
+      </c>
+      <c r="M12" t="s">
+        <v>133</v>
+      </c>
+      <c r="N12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O12">
+        <v>21</v>
+      </c>
+      <c r="P12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>517</v>
+      </c>
+      <c r="R12">
+        <v>32</v>
+      </c>
+      <c r="S12" t="s">
+        <v>518</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="U12" t="s">
+        <v>519</v>
+      </c>
+      <c r="V12" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W12" t="s">
+        <v>520</v>
+      </c>
+      <c r="X12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>521</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>523</v>
+      </c>
+      <c r="D13" t="s">
+        <v>153</v>
+      </c>
+      <c r="E13" t="s">
+        <v>130</v>
+      </c>
+      <c r="F13" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" t="s">
+        <v>131</v>
+      </c>
+      <c r="H13" t="s">
+        <v>144</v>
+      </c>
+      <c r="I13">
+        <v>5.6</v>
+      </c>
+      <c r="J13">
+        <v>7.2</v>
+      </c>
+      <c r="K13" t="s">
+        <v>440</v>
+      </c>
+      <c r="L13" t="s">
+        <v>441</v>
+      </c>
+      <c r="M13" t="s">
+        <v>133</v>
+      </c>
+      <c r="N13" t="s">
+        <v>38</v>
+      </c>
+      <c r="O13">
+        <v>9</v>
+      </c>
+      <c r="P13" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>524</v>
+      </c>
+      <c r="R13">
+        <v>50</v>
+      </c>
+      <c r="S13" t="s">
+        <v>525</v>
+      </c>
+      <c r="T13" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="U13" t="s">
+        <v>527</v>
+      </c>
+      <c r="V13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W13" t="s">
+        <v>528</v>
+      </c>
+      <c r="X13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>529</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>531</v>
+      </c>
+      <c r="D14" t="s">
+        <v>162</v>
+      </c>
+      <c r="E14" t="s">
+        <v>130</v>
+      </c>
+      <c r="F14" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" t="s">
+        <v>163</v>
+      </c>
+      <c r="H14" t="s">
+        <v>132</v>
+      </c>
+      <c r="I14">
+        <v>6.6</v>
+      </c>
+      <c r="J14">
+        <v>4.9</v>
+      </c>
+      <c r="K14" t="s">
+        <v>440</v>
+      </c>
+      <c r="L14" t="s">
+        <v>441</v>
+      </c>
+      <c r="M14" t="s">
+        <v>133</v>
+      </c>
+      <c r="N14" t="s">
+        <v>38</v>
+      </c>
+      <c r="O14">
+        <v>18</v>
+      </c>
+      <c r="P14" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>532</v>
+      </c>
+      <c r="R14">
+        <v>18</v>
+      </c>
+      <c r="S14" t="s">
+        <v>533</v>
+      </c>
+      <c r="T14" t="s">
+        <v>113</v>
+      </c>
+      <c r="U14" t="s">
+        <v>114</v>
+      </c>
+      <c r="V14" t="s">
+        <v>115</v>
+      </c>
+      <c r="W14" t="s">
+        <v>116</v>
+      </c>
+      <c r="X14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>534</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>536</v>
+      </c>
+      <c r="D15" t="s">
+        <v>172</v>
+      </c>
+      <c r="E15" t="s">
+        <v>130</v>
+      </c>
+      <c r="F15" t="s">
+        <v>60</v>
+      </c>
+      <c r="G15" t="s">
+        <v>131</v>
+      </c>
+      <c r="H15" t="s">
+        <v>163</v>
+      </c>
+      <c r="I15">
+        <v>7.7</v>
+      </c>
+      <c r="J15">
+        <v>7.6</v>
+      </c>
+      <c r="K15" t="s">
+        <v>440</v>
+      </c>
+      <c r="L15" t="s">
+        <v>441</v>
+      </c>
+      <c r="M15" t="s">
+        <v>133</v>
+      </c>
+      <c r="N15" t="s">
+        <v>38</v>
+      </c>
+      <c r="O15">
+        <v>12</v>
+      </c>
+      <c r="P15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>537</v>
+      </c>
+      <c r="R15">
+        <v>45</v>
+      </c>
+      <c r="S15" t="s">
+        <v>538</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="U15" t="s">
+        <v>539</v>
+      </c>
+      <c r="V15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W15" t="s">
+        <v>540</v>
+      </c>
+      <c r="X15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>541</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>543</v>
+      </c>
+      <c r="D16" t="s">
+        <v>181</v>
+      </c>
+      <c r="E16" t="s">
+        <v>130</v>
+      </c>
+      <c r="F16" t="s">
+        <v>60</v>
+      </c>
+      <c r="G16" t="s">
+        <v>34</v>
+      </c>
+      <c r="H16" t="s">
+        <v>132</v>
+      </c>
+      <c r="I16">
+        <v>11.3</v>
+      </c>
+      <c r="J16">
+        <v>13.3</v>
+      </c>
+      <c r="K16" t="s">
+        <v>440</v>
+      </c>
+      <c r="L16" t="s">
+        <v>441</v>
+      </c>
+      <c r="M16" t="s">
+        <v>133</v>
+      </c>
+      <c r="N16" t="s">
+        <v>38</v>
+      </c>
+      <c r="O16">
+        <v>25</v>
+      </c>
+      <c r="P16" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>544</v>
+      </c>
+      <c r="R16">
+        <v>35</v>
+      </c>
+      <c r="S16" t="s">
+        <v>545</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="U16" t="s">
+        <v>546</v>
+      </c>
+      <c r="V16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W16" t="s">
+        <v>547</v>
+      </c>
+      <c r="X16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>548</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>550</v>
+      </c>
+      <c r="D17" t="s">
+        <v>190</v>
+      </c>
+      <c r="E17" t="s">
+        <v>191</v>
+      </c>
+      <c r="F17" t="s">
+        <v>32</v>
+      </c>
+      <c r="G17" t="s">
+        <v>110</v>
+      </c>
+      <c r="H17" t="s">
+        <v>192</v>
+      </c>
+      <c r="I17">
+        <v>9.8</v>
+      </c>
+      <c r="J17">
+        <v>9.8</v>
+      </c>
+      <c r="K17" t="s">
+        <v>440</v>
+      </c>
+      <c r="L17" t="s">
+        <v>441</v>
+      </c>
+      <c r="M17" t="s">
+        <v>193</v>
+      </c>
+      <c r="N17" t="s">
+        <v>38</v>
+      </c>
+      <c r="O17">
+        <v>28</v>
+      </c>
+      <c r="P17" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>551</v>
+      </c>
+      <c r="R17">
+        <v>24</v>
+      </c>
+      <c r="S17" t="s">
+        <v>552</v>
+      </c>
+      <c r="T17" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="U17" t="s">
+        <v>553</v>
+      </c>
+      <c r="V17" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="W17" t="s">
+        <v>554</v>
+      </c>
+      <c r="X17" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>555</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" t="s">
+        <v>557</v>
+      </c>
+      <c r="D18" t="s">
+        <v>202</v>
+      </c>
+      <c r="E18" t="s">
+        <v>191</v>
+      </c>
+      <c r="F18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H18" t="s">
+        <v>192</v>
+      </c>
+      <c r="I18">
+        <v>4.4</v>
+      </c>
+      <c r="J18">
+        <v>4.4</v>
+      </c>
+      <c r="K18" t="s">
+        <v>440</v>
+      </c>
+      <c r="L18" t="s">
+        <v>441</v>
+      </c>
+      <c r="M18" t="s">
+        <v>193</v>
+      </c>
+      <c r="N18" t="s">
+        <v>38</v>
+      </c>
+      <c r="O18">
+        <v>12</v>
+      </c>
+      <c r="P18" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>558</v>
+      </c>
+      <c r="R18">
+        <v>10</v>
+      </c>
+      <c r="S18" t="s">
+        <v>559</v>
+      </c>
+      <c r="T18" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="U18" t="s">
+        <v>560</v>
+      </c>
+      <c r="V18" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="W18" t="s">
+        <v>561</v>
+      </c>
+      <c r="X18" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>562</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>564</v>
+      </c>
+      <c r="D19" t="s">
+        <v>210</v>
+      </c>
+      <c r="E19" t="s">
+        <v>191</v>
+      </c>
+      <c r="F19" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" t="s">
+        <v>110</v>
+      </c>
+      <c r="H19" t="s">
+        <v>211</v>
+      </c>
+      <c r="I19">
+        <v>8.9</v>
+      </c>
+      <c r="J19">
+        <v>8.8</v>
+      </c>
+      <c r="K19" t="s">
+        <v>440</v>
+      </c>
+      <c r="L19" t="s">
+        <v>441</v>
+      </c>
+      <c r="M19" t="s">
+        <v>193</v>
+      </c>
+      <c r="N19" t="s">
+        <v>38</v>
+      </c>
+      <c r="O19">
+        <v>23</v>
+      </c>
+      <c r="P19" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>565</v>
+      </c>
+      <c r="R19">
+        <v>22</v>
+      </c>
+      <c r="S19" t="s">
+        <v>566</v>
+      </c>
+      <c r="T19" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="U19" t="s">
+        <v>567</v>
+      </c>
+      <c r="V19" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="W19" t="s">
+        <v>568</v>
+      </c>
+      <c r="X19" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>569</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" t="s">
+        <v>571</v>
+      </c>
+      <c r="D20" t="s">
+        <v>219</v>
+      </c>
+      <c r="E20" t="s">
+        <v>220</v>
+      </c>
+      <c r="F20" t="s">
+        <v>32</v>
+      </c>
+      <c r="G20" t="s">
+        <v>221</v>
+      </c>
+      <c r="H20" t="s">
+        <v>222</v>
+      </c>
+      <c r="I20">
+        <v>7.9</v>
+      </c>
+      <c r="J20">
+        <v>7.8</v>
+      </c>
+      <c r="K20" t="s">
+        <v>440</v>
+      </c>
+      <c r="L20" t="s">
+        <v>441</v>
+      </c>
+      <c r="M20" t="s">
+        <v>223</v>
+      </c>
+      <c r="N20" t="s">
+        <v>38</v>
+      </c>
+      <c r="O20">
+        <v>17</v>
+      </c>
+      <c r="P20" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>572</v>
+      </c>
+      <c r="R20">
+        <v>26</v>
+      </c>
+      <c r="S20" t="s">
+        <v>573</v>
+      </c>
+      <c r="T20" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="U20" t="s">
+        <v>497</v>
+      </c>
+      <c r="V20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W20" t="s">
+        <v>498</v>
+      </c>
+      <c r="X20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>574</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" t="s">
+        <v>576</v>
+      </c>
+      <c r="D21" t="s">
+        <v>229</v>
+      </c>
+      <c r="E21" t="s">
+        <v>220</v>
+      </c>
+      <c r="F21" t="s">
+        <v>60</v>
+      </c>
+      <c r="G21" t="s">
+        <v>230</v>
+      </c>
+      <c r="H21" t="s">
+        <v>222</v>
+      </c>
+      <c r="I21">
+        <v>3.7</v>
+      </c>
+      <c r="J21">
+        <v>3.7</v>
+      </c>
+      <c r="K21" t="s">
+        <v>440</v>
+      </c>
+      <c r="L21" t="s">
+        <v>441</v>
+      </c>
+      <c r="M21" t="s">
+        <v>38</v>
+      </c>
+      <c r="N21" t="s">
+        <v>38</v>
+      </c>
+      <c r="O21">
+        <v>51</v>
+      </c>
+      <c r="P21" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>577</v>
+      </c>
+      <c r="R21">
+        <v>13</v>
+      </c>
+      <c r="S21" t="s">
+        <v>578</v>
+      </c>
+      <c r="T21" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="U21" t="s">
+        <v>580</v>
+      </c>
+      <c r="V21" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="W21" t="s">
+        <v>581</v>
+      </c>
+      <c r="X21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>582</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" t="s">
+        <v>584</v>
+      </c>
+      <c r="D22" t="s">
+        <v>238</v>
+      </c>
+      <c r="E22" t="s">
+        <v>220</v>
+      </c>
+      <c r="F22" t="s">
+        <v>60</v>
+      </c>
+      <c r="G22" t="s">
+        <v>221</v>
+      </c>
+      <c r="H22" t="s">
+        <v>230</v>
+      </c>
+      <c r="I22">
+        <v>4.1</v>
+      </c>
+      <c r="J22">
+        <v>4.1</v>
+      </c>
+      <c r="K22" t="s">
+        <v>440</v>
+      </c>
+      <c r="L22" t="s">
+        <v>441</v>
+      </c>
+      <c r="M22" t="s">
+        <v>38</v>
+      </c>
+      <c r="N22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O22">
+        <v>57</v>
+      </c>
+      <c r="P22" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>585</v>
+      </c>
+      <c r="R22">
+        <v>13</v>
+      </c>
+      <c r="S22" t="s">
+        <v>586</v>
+      </c>
+      <c r="T22" s="3" t="s">
+        <v>587</v>
+      </c>
+      <c r="U22" t="s">
+        <v>588</v>
+      </c>
+      <c r="V22" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="W22" t="s">
+        <v>589</v>
+      </c>
+      <c r="X22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>590</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" t="s">
+        <v>592</v>
+      </c>
+      <c r="D23" t="s">
+        <v>246</v>
+      </c>
+      <c r="E23" t="s">
+        <v>220</v>
+      </c>
+      <c r="F23" t="s">
+        <v>60</v>
+      </c>
+      <c r="G23" t="s">
+        <v>221</v>
+      </c>
+      <c r="H23" t="s">
+        <v>247</v>
+      </c>
+      <c r="I23">
+        <v>6.6</v>
+      </c>
+      <c r="J23">
+        <v>6.5</v>
+      </c>
+      <c r="K23" t="s">
+        <v>440</v>
+      </c>
+      <c r="L23" t="s">
+        <v>441</v>
+      </c>
+      <c r="M23" t="s">
+        <v>223</v>
+      </c>
+      <c r="N23" t="s">
+        <v>38</v>
+      </c>
+      <c r="O23">
+        <v>14</v>
+      </c>
+      <c r="P23" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>593</v>
+      </c>
+      <c r="R23">
+        <v>23</v>
+      </c>
+      <c r="S23" t="s">
+        <v>422</v>
+      </c>
+      <c r="T23" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="U23" t="s">
+        <v>423</v>
+      </c>
+      <c r="V23" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W23" t="s">
+        <v>424</v>
+      </c>
+      <c r="X23" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>594</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" t="s">
+        <v>596</v>
+      </c>
+      <c r="D24" t="s">
+        <v>255</v>
+      </c>
+      <c r="E24" t="s">
+        <v>220</v>
+      </c>
+      <c r="F24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" t="s">
+        <v>230</v>
+      </c>
+      <c r="H24" t="s">
+        <v>247</v>
+      </c>
+      <c r="I24">
+        <v>2.4</v>
+      </c>
+      <c r="J24">
+        <v>2.4</v>
+      </c>
+      <c r="K24" t="s">
+        <v>440</v>
+      </c>
+      <c r="L24" t="s">
+        <v>441</v>
+      </c>
+      <c r="M24" t="s">
+        <v>38</v>
+      </c>
+      <c r="N24" t="s">
+        <v>38</v>
+      </c>
+      <c r="O24">
+        <v>33</v>
+      </c>
+      <c r="P24" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>597</v>
+      </c>
+      <c r="R24">
+        <v>10</v>
+      </c>
+      <c r="S24" t="s">
+        <v>598</v>
+      </c>
+      <c r="T24" s="3" t="s">
+        <v>599</v>
+      </c>
+      <c r="U24" t="s">
+        <v>600</v>
+      </c>
+      <c r="V24" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="W24" t="s">
+        <v>601</v>
+      </c>
+      <c r="X24" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>602</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>604</v>
+      </c>
+      <c r="D25" t="s">
+        <v>263</v>
+      </c>
+      <c r="E25" t="s">
+        <v>220</v>
+      </c>
+      <c r="F25" t="s">
+        <v>60</v>
+      </c>
+      <c r="G25" t="s">
+        <v>247</v>
+      </c>
+      <c r="H25" t="s">
+        <v>222</v>
+      </c>
+      <c r="I25">
+        <v>1.3</v>
+      </c>
+      <c r="J25">
+        <v>1.3</v>
+      </c>
+      <c r="K25" t="s">
+        <v>440</v>
+      </c>
+      <c r="L25" t="s">
+        <v>441</v>
+      </c>
+      <c r="M25" t="s">
+        <v>38</v>
+      </c>
+      <c r="N25" t="s">
+        <v>38</v>
+      </c>
+      <c r="O25">
+        <v>18</v>
+      </c>
+      <c r="P25" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>605</v>
+      </c>
+      <c r="R25">
+        <v>3</v>
+      </c>
+      <c r="S25" t="s">
+        <v>606</v>
+      </c>
+      <c r="T25" s="3" t="s">
+        <v>607</v>
+      </c>
+      <c r="U25" t="s">
+        <v>608</v>
+      </c>
+      <c r="V25" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="W25" t="s">
+        <v>609</v>
+      </c>
+      <c r="X25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>610</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>611</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AA1"/>
+  <hyperlinks>
+    <hyperlink ref="X2" r:id="rId1"/>
+    <hyperlink ref="Y2" r:id="rId2"/>
+    <hyperlink ref="X3" r:id="rId3"/>
+    <hyperlink ref="Y3" r:id="rId4"/>
+    <hyperlink ref="X4" r:id="rId5"/>
+    <hyperlink ref="Y4" r:id="rId6"/>
+    <hyperlink ref="X5" r:id="rId7"/>
+    <hyperlink ref="Y5" r:id="rId8"/>
+    <hyperlink ref="X6" r:id="rId9"/>
+    <hyperlink ref="Y6" r:id="rId10"/>
+    <hyperlink ref="X7" r:id="rId11"/>
+    <hyperlink ref="Y7" r:id="rId12"/>
+    <hyperlink ref="X8" r:id="rId13"/>
+    <hyperlink ref="Y8" r:id="rId14"/>
+    <hyperlink ref="X9" r:id="rId15"/>
+    <hyperlink ref="Y9" r:id="rId16"/>
+    <hyperlink ref="X10" r:id="rId17"/>
+    <hyperlink ref="Y10" r:id="rId18"/>
+    <hyperlink ref="X11" r:id="rId19"/>
+    <hyperlink ref="Y11" r:id="rId20"/>
+    <hyperlink ref="X12" r:id="rId21"/>
+    <hyperlink ref="Y12" r:id="rId22"/>
+    <hyperlink ref="X13" r:id="rId23"/>
+    <hyperlink ref="Y13" r:id="rId24"/>
+    <hyperlink ref="X14" r:id="rId25"/>
+    <hyperlink ref="Y14" r:id="rId26"/>
+    <hyperlink ref="X15" r:id="rId27"/>
+    <hyperlink ref="Y15" r:id="rId28"/>
+    <hyperlink ref="X16" r:id="rId29"/>
+    <hyperlink ref="Y16" r:id="rId30"/>
+    <hyperlink ref="X17" r:id="rId31"/>
+    <hyperlink ref="Y17" r:id="rId32"/>
+    <hyperlink ref="X18" r:id="rId33"/>
+    <hyperlink ref="Y18" r:id="rId34"/>
+    <hyperlink ref="X19" r:id="rId35"/>
+    <hyperlink ref="Y19" r:id="rId36"/>
+    <hyperlink ref="X20" r:id="rId37"/>
+    <hyperlink ref="Y20" r:id="rId38"/>
+    <hyperlink ref="X21" r:id="rId39"/>
+    <hyperlink ref="Y21" r:id="rId40"/>
+    <hyperlink ref="X22" r:id="rId41"/>
+    <hyperlink ref="Y22" r:id="rId42"/>
+    <hyperlink ref="X23" r:id="rId43"/>
+    <hyperlink ref="Y23" r:id="rId44"/>
+    <hyperlink ref="X24" r:id="rId45"/>
+    <hyperlink ref="Y24" r:id="rId46"/>
+    <hyperlink ref="X25" r:id="rId47"/>
+    <hyperlink ref="Y25" r:id="rId48"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AG25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:33" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>3</v>
       </c>
@@ -6087,61 +8774,88 @@
         <v>9</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>439</v>
+        <v>612</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>440</v>
+        <v>613</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>441</v>
+        <v>614</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>442</v>
+        <v>615</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>443</v>
+        <v>616</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>444</v>
+        <v>617</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>445</v>
+        <v>618</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>446</v>
+        <v>619</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>447</v>
+        <v>620</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>448</v>
+        <v>621</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>449</v>
+        <v>622</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>450</v>
+        <v>623</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>451</v>
+        <v>624</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>452</v>
+        <v>625</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>453</v>
+        <v>626</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>454</v>
+        <v>627</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>455</v>
+        <v>628</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>456</v>
+        <v>629</v>
+      </c>
+      <c r="Y1" s="4" t="s">
+        <v>630</v>
+      </c>
+      <c r="Z1" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="AA1" s="4" t="s">
+        <v>632</v>
+      </c>
+      <c r="AB1" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="AC1" s="4" t="s">
+        <v>634</v>
+      </c>
+      <c r="AD1" s="4" t="s">
+        <v>635</v>
+      </c>
+      <c r="AE1" s="4" t="s">
+        <v>636</v>
+      </c>
+      <c r="AF1" s="4" t="s">
+        <v>637</v>
+      </c>
+      <c r="AG1" s="4" t="s">
+        <v>638</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -6214,8 +8928,35 @@
       <c r="X2" t="s">
         <v>277</v>
       </c>
+      <c r="Y2" t="s">
+        <v>439</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB2">
+        <v>31</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>442</v>
+      </c>
+      <c r="AE2">
+        <v>58</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>446</v>
+      </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -6288,8 +9029,35 @@
       <c r="X3" t="s">
         <v>285</v>
       </c>
+      <c r="Y3" t="s">
+        <v>449</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB3">
+        <v>30</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>450</v>
+      </c>
+      <c r="AE3">
+        <v>65</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>454</v>
+      </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -6362,8 +9130,35 @@
       <c r="X4" t="s">
         <v>293</v>
       </c>
+      <c r="Y4" t="s">
+        <v>457</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB4">
+        <v>54</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>639</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>458</v>
+      </c>
+      <c r="AE4">
+        <v>18</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>138</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>462</v>
+      </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -6436,8 +9231,35 @@
       <c r="X5" t="s">
         <v>300</v>
       </c>
+      <c r="Y5" t="s">
+        <v>465</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB5">
+        <v>11</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>466</v>
+      </c>
+      <c r="AE5">
+        <v>39</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>470</v>
+      </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>80</v>
       </c>
@@ -6510,8 +9332,35 @@
       <c r="X6" t="s">
         <v>306</v>
       </c>
+      <c r="Y6" t="s">
+        <v>473</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB6">
+        <v>11</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>474</v>
+      </c>
+      <c r="AE6">
+        <v>24</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>478</v>
+      </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>90</v>
       </c>
@@ -6584,8 +9433,35 @@
       <c r="X7" t="s">
         <v>314</v>
       </c>
+      <c r="Y7" t="s">
+        <v>481</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB7">
+        <v>15</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>482</v>
+      </c>
+      <c r="AE7">
+        <v>28</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>484</v>
+      </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>99</v>
       </c>
@@ -6658,8 +9534,35 @@
       <c r="X8" t="s">
         <v>321</v>
       </c>
+      <c r="Y8" t="s">
+        <v>487</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB8">
+        <v>23</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD8" t="s">
+        <v>488</v>
+      </c>
+      <c r="AE8">
+        <v>31</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG8" t="s">
+        <v>491</v>
+      </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>109</v>
       </c>
@@ -6732,8 +9635,35 @@
       <c r="X9" t="s">
         <v>328</v>
       </c>
+      <c r="Y9" t="s">
+        <v>494</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB9">
+        <v>17</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>495</v>
+      </c>
+      <c r="AE9">
+        <v>26</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG9" t="s">
+        <v>498</v>
+      </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>120</v>
       </c>
@@ -6806,8 +9736,35 @@
       <c r="X10" t="s">
         <v>336</v>
       </c>
+      <c r="Y10" t="s">
+        <v>501</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB10">
+        <v>16</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>502</v>
+      </c>
+      <c r="AE10">
+        <v>49</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>506</v>
+      </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>129</v>
       </c>
@@ -6880,8 +9837,35 @@
       <c r="X11" t="s">
         <v>344</v>
       </c>
+      <c r="Y11" t="s">
+        <v>509</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>133</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB11">
+        <v>30</v>
+      </c>
+      <c r="AC11" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD11" t="s">
+        <v>510</v>
+      </c>
+      <c r="AE11">
+        <v>58</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG11" t="s">
+        <v>513</v>
+      </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>143</v>
       </c>
@@ -6954,8 +9938,35 @@
       <c r="X12" t="s">
         <v>95</v>
       </c>
+      <c r="Y12" t="s">
+        <v>516</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>133</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB12">
+        <v>21</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD12" t="s">
+        <v>517</v>
+      </c>
+      <c r="AE12">
+        <v>32</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG12" t="s">
+        <v>520</v>
+      </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>153</v>
       </c>
@@ -7028,8 +10039,35 @@
       <c r="X13" t="s">
         <v>357</v>
       </c>
+      <c r="Y13" t="s">
+        <v>523</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>133</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB13">
+        <v>9</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>524</v>
+      </c>
+      <c r="AE13">
+        <v>50</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG13" t="s">
+        <v>528</v>
+      </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>162</v>
       </c>
@@ -7102,8 +10140,35 @@
       <c r="X14" t="s">
         <v>364</v>
       </c>
+      <c r="Y14" t="s">
+        <v>531</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>133</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB14">
+        <v>18</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>532</v>
+      </c>
+      <c r="AE14">
+        <v>18</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG14" t="s">
+        <v>116</v>
+      </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>172</v>
       </c>
@@ -7176,8 +10241,35 @@
       <c r="X15" t="s">
         <v>371</v>
       </c>
+      <c r="Y15" t="s">
+        <v>536</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>133</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB15">
+        <v>12</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD15" t="s">
+        <v>537</v>
+      </c>
+      <c r="AE15">
+        <v>45</v>
+      </c>
+      <c r="AF15" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG15" t="s">
+        <v>540</v>
+      </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>181</v>
       </c>
@@ -7250,8 +10342,35 @@
       <c r="X16" t="s">
         <v>378</v>
       </c>
+      <c r="Y16" t="s">
+        <v>543</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>133</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB16">
+        <v>25</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD16" t="s">
+        <v>544</v>
+      </c>
+      <c r="AE16">
+        <v>35</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG16" t="s">
+        <v>547</v>
+      </c>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>190</v>
       </c>
@@ -7324,8 +10443,35 @@
       <c r="X17" t="s">
         <v>386</v>
       </c>
+      <c r="Y17" t="s">
+        <v>550</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>193</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB17">
+        <v>28</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD17" t="s">
+        <v>551</v>
+      </c>
+      <c r="AE17">
+        <v>24</v>
+      </c>
+      <c r="AF17" t="s">
+        <v>138</v>
+      </c>
+      <c r="AG17" t="s">
+        <v>554</v>
+      </c>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>202</v>
       </c>
@@ -7398,8 +10544,35 @@
       <c r="X18" t="s">
         <v>259</v>
       </c>
+      <c r="Y18" t="s">
+        <v>557</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>193</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB18">
+        <v>12</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>558</v>
+      </c>
+      <c r="AE18">
+        <v>10</v>
+      </c>
+      <c r="AF18" t="s">
+        <v>138</v>
+      </c>
+      <c r="AG18" t="s">
+        <v>561</v>
+      </c>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>210</v>
       </c>
@@ -7472,8 +10645,35 @@
       <c r="X19" t="s">
         <v>398</v>
       </c>
+      <c r="Y19" t="s">
+        <v>564</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>193</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB19">
+        <v>23</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>565</v>
+      </c>
+      <c r="AE19">
+        <v>22</v>
+      </c>
+      <c r="AF19" t="s">
+        <v>138</v>
+      </c>
+      <c r="AG19" t="s">
+        <v>568</v>
+      </c>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>219</v>
       </c>
@@ -7546,8 +10746,35 @@
       <c r="X20" t="s">
         <v>405</v>
       </c>
+      <c r="Y20" t="s">
+        <v>571</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>223</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB20">
+        <v>17</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>572</v>
+      </c>
+      <c r="AE20">
+        <v>26</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG20" t="s">
+        <v>498</v>
+      </c>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>229</v>
       </c>
@@ -7620,8 +10847,35 @@
       <c r="X21" t="s">
         <v>412</v>
       </c>
+      <c r="Y21" t="s">
+        <v>576</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB21">
+        <v>51</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>639</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>577</v>
+      </c>
+      <c r="AE21">
+        <v>13</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>138</v>
+      </c>
+      <c r="AG21" t="s">
+        <v>581</v>
+      </c>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>238</v>
       </c>
@@ -7694,8 +10948,35 @@
       <c r="X22" t="s">
         <v>177</v>
       </c>
+      <c r="Y22" t="s">
+        <v>584</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB22">
+        <v>57</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>639</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>585</v>
+      </c>
+      <c r="AE22">
+        <v>13</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>138</v>
+      </c>
+      <c r="AG22" t="s">
+        <v>589</v>
+      </c>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>246</v>
       </c>
@@ -7768,8 +11049,35 @@
       <c r="X23" t="s">
         <v>424</v>
       </c>
+      <c r="Y23" t="s">
+        <v>592</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>223</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB23">
+        <v>14</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>593</v>
+      </c>
+      <c r="AE23">
+        <v>23</v>
+      </c>
+      <c r="AF23" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG23" t="s">
+        <v>424</v>
+      </c>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>255</v>
       </c>
@@ -7842,8 +11150,35 @@
       <c r="X24" t="s">
         <v>431</v>
       </c>
+      <c r="Y24" t="s">
+        <v>596</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB24">
+        <v>33</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>639</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>597</v>
+      </c>
+      <c r="AE24">
+        <v>10</v>
+      </c>
+      <c r="AF24" t="s">
+        <v>138</v>
+      </c>
+      <c r="AG24" t="s">
+        <v>601</v>
+      </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>263</v>
       </c>
@@ -7916,9 +11251,36 @@
       <c r="X25" t="s">
         <v>116</v>
       </c>
+      <c r="Y25" t="s">
+        <v>604</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB25">
+        <v>18</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>639</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>605</v>
+      </c>
+      <c r="AE25">
+        <v>3</v>
+      </c>
+      <c r="AF25" t="s">
+        <v>138</v>
+      </c>
+      <c r="AG25" t="s">
+        <v>609</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X1"/>
+  <autoFilter ref="A1:AG1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
🔄 Auto-collect traffic data: 2026-09-29 07:09 PM IST
</commit_message>
<xml_diff>
--- a/output/excel/Metro_vs_Car_Data_2026-09-29_Tue.xlsx
+++ b/output/excel/Metro_vs_Car_Data_2026-09-29_Tue.xlsx
@@ -7,14 +7,15 @@
     <sheet sheetId="1" name="12_00 AM" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="10_00 AM" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="1_00 PM" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="All Periods Combined" state="visible" r:id="rId7"/>
+    <sheet sheetId="4" name="7_00 PM" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="All Periods Combined" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2370" uniqueCount="640">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3126" uniqueCount="807">
   <si>
     <t>Date</t>
   </si>
@@ -1852,6 +1853,480 @@
     <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/1_00_PM/MC-24/car.jpg</t>
   </si>
   <si>
+    <t>9/29/2026, 7:02:46 PM</t>
+  </si>
+  <si>
+    <t>7:00 PM</t>
+  </si>
+  <si>
+    <t>Tuesday (Weekday) - Evening Peak</t>
+  </si>
+  <si>
+    <t> | 28 min | 7:18 AM—7:46 AM | Blue Line | 7:18 AM from Dakshineswar | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 52 min | 12.4 km | via Barrackpore Trunk Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.86x</t>
+  </si>
+  <si>
+    <t>46.2% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-01/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-01/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:03:03 PM</t>
+  </si>
+  <si>
+    <t> | 29 min | 7:00 AM—7:29 AM | Blue Line | 7:00 AM from Shahid Khudiram | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 1 hr 8 min | 14.7 km | via Netaji Subhas Chandra Bose Rd | Fastest route, despite heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>39 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.34x</t>
+  </si>
+  <si>
+    <t>57.4% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-02/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-02/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:03:20 PM</t>
+  </si>
+  <si>
+    <t> | 8 min | 7:01 AM—7:09 AM | Blue Line | 7:01 AM from Shyambazar | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>2.25x</t>
+  </si>
+  <si>
+    <t>55.6% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-03/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-03/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:03:37 PM</t>
+  </si>
+  <si>
+    <t> | 11 min | 7:00 AM—7:11 AM | Blue Line | 7:00 AM from Shyambazar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 31 min | 5.2 km | via Jatindra Mohan Ave and Central Ave/Chittaranjan Ave | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>20 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.82x</t>
+  </si>
+  <si>
+    <t>64.5% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-04/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-04/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:03:53 PM</t>
+  </si>
+  <si>
+    <t> | 11 min | 7:09 AM—7:20 AM | Blue Line | 7:09 AM from Kalighat | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 28 min | 5.1 km | via Shyama Prasad Mukherjee Rd and Ashutosh Mukherjee Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>17 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.55x</t>
+  </si>
+  <si>
+    <t>60.7% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-05/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-05/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:04:11 PM</t>
+  </si>
+  <si>
+    <t> | 12 min | 7:18 AM—7:30 AM | Blue Line | 7:18 AM from Dakshineswar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 26 min | 7.0 km | via Barrackpore Trunk Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-06/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-06/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:04:28 PM</t>
+  </si>
+  <si>
+    <t> | 18 min | 7:11 AM—7:29 AM | Blue Line | 7:11 AM from Esplanade | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 40 min | 8.3 km | via Chowringee Rd/Jawaharlal Nehru Rd and Ashutosh Mukherjee Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>2.22x</t>
+  </si>
+  <si>
+    <t>55.0% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-07/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-07/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:04:44 PM</t>
+  </si>
+  <si>
+    <t> | 15 min | 7:01 AM—7:16 AM | Blue Line | 7:01 AM from Mahanayak Uttam Kumar | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 32 min | 6.4 km | via Netaji Subhas Chandra Bose Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>2.13x</t>
+  </si>
+  <si>
+    <t>53.1% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-08/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-08/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:05:01 PM</t>
+  </si>
+  <si>
+    <t> | 16 min | 7:09 AM—7:25 AM | Blue Line | 7:09 AM from Dumdum | ₹15.00 | Details</t>
+  </si>
+  <si>
+    <t> | 46 min | 8.8 km | via Jessore Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>30 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.88x</t>
+  </si>
+  <si>
+    <t>65.2% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-09/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-09/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:05:19 PM</t>
+  </si>
+  <si>
+    <t> | 30 min | 7:02 AM—7:32 AM | Green Line | 7:02 AM from Howrah | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t> | 1 hr 6 min | 11.7 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>36 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>2.20x</t>
+  </si>
+  <si>
+    <t>54.5% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-10/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-10/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:05:37 PM</t>
+  </si>
+  <si>
+    <t> | 21 min | 7:11 AM—7:32 AM | Green Line | 7:11 AM from Sealdah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 33 min | 7.9 km | via Beleghata Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-11/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-11/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:05:54 PM</t>
+  </si>
+  <si>
+    <t> | 9 min | 7:02 AM—7:11 AM | Green Line | 7:02 AM from Howrah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 52 min | 7.2 km | via Kali Krishna Tagore St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>43 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>5.78x</t>
+  </si>
+  <si>
+    <t>82.7% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-12/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-12/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:06:12 PM</t>
+  </si>
+  <si>
+    <t> | 18 min | 7:14 AM—7:32 AM | Green Line | 7:14 AM from Phoolbagan | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-13/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-13/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:06:28 PM</t>
+  </si>
+  <si>
+    <t> | 12 min | 7:02 AM—7:14 AM | Green Line | 7:02 AM from Howrah | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 56 min | 7.6 km | via Kali Krishna Tagore St | Fastest route, despite much heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>44 min (Metro Faster)</t>
+  </si>
+  <si>
+    <t>4.67x</t>
+  </si>
+  <si>
+    <t>78.6% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-14/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-14/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:06:46 PM</t>
+  </si>
+  <si>
+    <t> | 25 min | 7:07 AM—7:32 AM | Green Line | 7:07 AM from Esplanade | ₹30.00 | Details</t>
+  </si>
+  <si>
+    <t> | 39 min | 13.3 km | via Indira Gandhi Sarani and Park St | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.56x</t>
+  </si>
+  <si>
+    <t>35.9% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-15/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-15/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:07:03 PM</t>
+  </si>
+  <si>
+    <t> | 28 min | 9.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route, the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-16/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-16/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:07:21 PM</t>
+  </si>
+  <si>
+    <t> | 17 min | 7:51 AM—8:08 AM | Orange Line | 7:51 AM from Hemanta Mukhopadhyay | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t> | 11 min | 4.4 km | via Bangaon - Kulpi Rd/Biswa Bangla Sarani/Eastern Metropolitan Bypass/Thakurnagar - Panchpota Rd | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>0.65x</t>
+  </si>
+  <si>
+    <t>35.3% (vs Metro)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-17/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-17/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:07:38 PM</t>
+  </si>
+  <si>
+    <t> | 26 min | 8.8 km | via New Garia Sta Rd/Panchasyar Main Rd | Fastest route now due to traffic conditions | Details | Preview</t>
+  </si>
+  <si>
+    <t>11.5% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-18/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-18/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:07:55 PM</t>
+  </si>
+  <si>
+    <t> | 17 min | 7:03 AM—7:20 AM | Purple Line | 7:03 AM from Joka | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 29 min | 7.8 km | via NH 12 | Fastest route, lighter traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.71x</t>
+  </si>
+  <si>
+    <t>41.4% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-19/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-19/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:08:12 PM</t>
+  </si>
+  <si>
+    <t> | 9 min | 7:11 AM—7:20 AM | Purple Line | 7:11 AM from Behala Chowrasta | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t> | 16 min | 3.7 km | via NH 12 | Fastest route, despite heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>1.78x</t>
+  </si>
+  <si>
+    <t>43.8% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-20/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-20/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:08:29 PM</t>
+  </si>
+  <si>
+    <t> | 8 min | 7:03 AM—7:11 AM | Purple Line | 7:03 AM from Joka | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>1.63x</t>
+  </si>
+  <si>
+    <t>38.5% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-21/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-21/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:08:46 PM</t>
+  </si>
+  <si>
+    <t> | 14 min | 7:03 AM—7:17 AM | Purple Line | 7:03 AM from Joka | ₹20.00 | Details</t>
+  </si>
+  <si>
+    <t> | 22 min | 6.5 km | via NH 12 | Fastest route, despite the usual traffic | Details | Preview</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-22/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-22/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:09:03 PM</t>
+  </si>
+  <si>
+    <t> | 6 min | 7:11 AM—7:17 AM | Purple Line | 7:11 AM from Behala Chowrasta | ₹10.00 | Details</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-23/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-23/car.jpg</t>
+  </si>
+  <si>
+    <t>9/29/2026, 7:09:19 PM</t>
+  </si>
+  <si>
+    <t> | 3 min | 7:17 AM—7:20 AM | Purple Line | 7:17 AM from Taratala | ₹5.00 | Details</t>
+  </si>
+  <si>
+    <t> | 6 min | 1.3 km | via NH 12 | Fastest route, despite heavier traffic than usual | Details | Preview</t>
+  </si>
+  <si>
+    <t>2.00x</t>
+  </si>
+  <si>
+    <t>50.0% (vs Car)</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-24/metro.jpg</t>
+  </si>
+  <si>
+    <t>/home/runner/work/Metro-Traffic-Automation/Metro-Traffic-Automation/output/screenshots/2026-09-29/7_00_PM/MC-24/car.jpg</t>
+  </si>
+  <si>
     <t>12:00 AM Scraped At</t>
   </si>
   <si>
@@ -1931,6 +2406,33 @@
   </si>
   <si>
     <t>1:00 PM Savings (%)</t>
+  </si>
+  <si>
+    <t>7:00 PM Scraped At</t>
+  </si>
+  <si>
+    <t>7:00 PM Actual Metro</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro Walk</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro (min)</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro Route</t>
+  </si>
+  <si>
+    <t>7:00 PM Metro Raw Details</t>
+  </si>
+  <si>
+    <t>7:00 PM Car (min)</t>
+  </si>
+  <si>
+    <t>7:00 PM Faster Mode</t>
+  </si>
+  <si>
+    <t>7:00 PM Savings (%)</t>
   </si>
   <si>
     <t/>
@@ -8751,10 +9253,2147 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AG25"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:33" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>612</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2">
+        <v>15</v>
+      </c>
+      <c r="J2">
+        <v>12.4</v>
+      </c>
+      <c r="K2" t="s">
+        <v>613</v>
+      </c>
+      <c r="L2" t="s">
+        <v>614</v>
+      </c>
+      <c r="M2" t="s">
+        <v>37</v>
+      </c>
+      <c r="N2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O2">
+        <v>28</v>
+      </c>
+      <c r="P2" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>615</v>
+      </c>
+      <c r="R2">
+        <v>52</v>
+      </c>
+      <c r="S2" t="s">
+        <v>616</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="U2" t="s">
+        <v>617</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W2" t="s">
+        <v>618</v>
+      </c>
+      <c r="X2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>619</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>621</v>
+      </c>
+      <c r="D3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" t="s">
+        <v>50</v>
+      </c>
+      <c r="H3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3">
+        <v>14.9</v>
+      </c>
+      <c r="J3">
+        <v>14.7</v>
+      </c>
+      <c r="K3" t="s">
+        <v>613</v>
+      </c>
+      <c r="L3" t="s">
+        <v>614</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3">
+        <v>29</v>
+      </c>
+      <c r="P3" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>622</v>
+      </c>
+      <c r="R3">
+        <v>68</v>
+      </c>
+      <c r="S3" t="s">
+        <v>623</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="U3" t="s">
+        <v>625</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W3" t="s">
+        <v>626</v>
+      </c>
+      <c r="X3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>627</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>629</v>
+      </c>
+      <c r="D4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H4" t="s">
+        <v>62</v>
+      </c>
+      <c r="I4">
+        <v>3.8</v>
+      </c>
+      <c r="J4">
+        <v>3.5</v>
+      </c>
+      <c r="K4" t="s">
+        <v>613</v>
+      </c>
+      <c r="L4" t="s">
+        <v>614</v>
+      </c>
+      <c r="M4" t="s">
+        <v>37</v>
+      </c>
+      <c r="N4" t="s">
+        <v>38</v>
+      </c>
+      <c r="O4">
+        <v>8</v>
+      </c>
+      <c r="P4" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>630</v>
+      </c>
+      <c r="R4">
+        <v>18</v>
+      </c>
+      <c r="S4" t="s">
+        <v>459</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="U4" t="s">
+        <v>631</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W4" t="s">
+        <v>632</v>
+      </c>
+      <c r="X4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>633</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>635</v>
+      </c>
+      <c r="D5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5">
+        <v>5.1</v>
+      </c>
+      <c r="J5">
+        <v>5.2</v>
+      </c>
+      <c r="K5" t="s">
+        <v>613</v>
+      </c>
+      <c r="L5" t="s">
+        <v>614</v>
+      </c>
+      <c r="M5" t="s">
+        <v>37</v>
+      </c>
+      <c r="N5" t="s">
+        <v>38</v>
+      </c>
+      <c r="O5">
+        <v>11</v>
+      </c>
+      <c r="P5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>636</v>
+      </c>
+      <c r="R5">
+        <v>31</v>
+      </c>
+      <c r="S5" t="s">
+        <v>637</v>
+      </c>
+      <c r="T5" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="U5" t="s">
+        <v>639</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W5" t="s">
+        <v>640</v>
+      </c>
+      <c r="X5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>641</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" t="s">
+        <v>643</v>
+      </c>
+      <c r="D6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I6">
+        <v>5.2</v>
+      </c>
+      <c r="J6">
+        <v>5.1</v>
+      </c>
+      <c r="K6" t="s">
+        <v>613</v>
+      </c>
+      <c r="L6" t="s">
+        <v>614</v>
+      </c>
+      <c r="M6" t="s">
+        <v>37</v>
+      </c>
+      <c r="N6" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6">
+        <v>11</v>
+      </c>
+      <c r="P6" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>644</v>
+      </c>
+      <c r="R6">
+        <v>28</v>
+      </c>
+      <c r="S6" t="s">
+        <v>645</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="U6" t="s">
+        <v>647</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W6" t="s">
+        <v>648</v>
+      </c>
+      <c r="X6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>649</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>651</v>
+      </c>
+      <c r="D7" t="s">
+        <v>90</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>62</v>
+      </c>
+      <c r="I7">
+        <v>6.2</v>
+      </c>
+      <c r="J7">
+        <v>7</v>
+      </c>
+      <c r="K7" t="s">
+        <v>613</v>
+      </c>
+      <c r="L7" t="s">
+        <v>614</v>
+      </c>
+      <c r="M7" t="s">
+        <v>37</v>
+      </c>
+      <c r="N7" t="s">
+        <v>38</v>
+      </c>
+      <c r="O7">
+        <v>12</v>
+      </c>
+      <c r="P7" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>652</v>
+      </c>
+      <c r="R7">
+        <v>26</v>
+      </c>
+      <c r="S7" t="s">
+        <v>653</v>
+      </c>
+      <c r="T7" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="U7" t="s">
+        <v>453</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W7" t="s">
+        <v>454</v>
+      </c>
+      <c r="X7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>654</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
+        <v>656</v>
+      </c>
+      <c r="D8" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" t="s">
+        <v>100</v>
+      </c>
+      <c r="I8">
+        <v>7.8</v>
+      </c>
+      <c r="J8">
+        <v>8.3</v>
+      </c>
+      <c r="K8" t="s">
+        <v>613</v>
+      </c>
+      <c r="L8" t="s">
+        <v>614</v>
+      </c>
+      <c r="M8" t="s">
+        <v>37</v>
+      </c>
+      <c r="N8" t="s">
+        <v>38</v>
+      </c>
+      <c r="O8">
+        <v>18</v>
+      </c>
+      <c r="P8" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>657</v>
+      </c>
+      <c r="R8">
+        <v>40</v>
+      </c>
+      <c r="S8" t="s">
+        <v>658</v>
+      </c>
+      <c r="T8" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="U8" t="s">
+        <v>659</v>
+      </c>
+      <c r="V8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W8" t="s">
+        <v>660</v>
+      </c>
+      <c r="X8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>661</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>663</v>
+      </c>
+      <c r="D9" t="s">
+        <v>109</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" t="s">
+        <v>100</v>
+      </c>
+      <c r="H9" t="s">
+        <v>110</v>
+      </c>
+      <c r="I9">
+        <v>7.1</v>
+      </c>
+      <c r="J9">
+        <v>6.4</v>
+      </c>
+      <c r="K9" t="s">
+        <v>613</v>
+      </c>
+      <c r="L9" t="s">
+        <v>614</v>
+      </c>
+      <c r="M9" t="s">
+        <v>37</v>
+      </c>
+      <c r="N9" t="s">
+        <v>38</v>
+      </c>
+      <c r="O9">
+        <v>15</v>
+      </c>
+      <c r="P9" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>664</v>
+      </c>
+      <c r="R9">
+        <v>32</v>
+      </c>
+      <c r="S9" t="s">
+        <v>665</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="U9" t="s">
+        <v>666</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W9" t="s">
+        <v>667</v>
+      </c>
+      <c r="X9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>668</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" t="s">
+        <v>670</v>
+      </c>
+      <c r="D10" t="s">
+        <v>120</v>
+      </c>
+      <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" t="s">
+        <v>62</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+      <c r="I10">
+        <v>8.8</v>
+      </c>
+      <c r="J10">
+        <v>8.8</v>
+      </c>
+      <c r="K10" t="s">
+        <v>613</v>
+      </c>
+      <c r="L10" t="s">
+        <v>614</v>
+      </c>
+      <c r="M10" t="s">
+        <v>37</v>
+      </c>
+      <c r="N10" t="s">
+        <v>38</v>
+      </c>
+      <c r="O10">
+        <v>16</v>
+      </c>
+      <c r="P10" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>671</v>
+      </c>
+      <c r="R10">
+        <v>46</v>
+      </c>
+      <c r="S10" t="s">
+        <v>672</v>
+      </c>
+      <c r="T10" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="U10" t="s">
+        <v>674</v>
+      </c>
+      <c r="V10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W10" t="s">
+        <v>675</v>
+      </c>
+      <c r="X10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>676</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="s">
+        <v>678</v>
+      </c>
+      <c r="D11" t="s">
+        <v>129</v>
+      </c>
+      <c r="E11" t="s">
+        <v>130</v>
+      </c>
+      <c r="F11" t="s">
+        <v>32</v>
+      </c>
+      <c r="G11" t="s">
+        <v>131</v>
+      </c>
+      <c r="H11" t="s">
+        <v>132</v>
+      </c>
+      <c r="I11">
+        <v>14.2</v>
+      </c>
+      <c r="J11">
+        <v>11.7</v>
+      </c>
+      <c r="K11" t="s">
+        <v>613</v>
+      </c>
+      <c r="L11" t="s">
+        <v>614</v>
+      </c>
+      <c r="M11" t="s">
+        <v>133</v>
+      </c>
+      <c r="N11" t="s">
+        <v>38</v>
+      </c>
+      <c r="O11">
+        <v>30</v>
+      </c>
+      <c r="P11" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>679</v>
+      </c>
+      <c r="R11">
+        <v>66</v>
+      </c>
+      <c r="S11" t="s">
+        <v>680</v>
+      </c>
+      <c r="T11" s="2" t="s">
+        <v>681</v>
+      </c>
+      <c r="U11" t="s">
+        <v>682</v>
+      </c>
+      <c r="V11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W11" t="s">
+        <v>683</v>
+      </c>
+      <c r="X11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>684</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" t="s">
+        <v>686</v>
+      </c>
+      <c r="D12" t="s">
+        <v>143</v>
+      </c>
+      <c r="E12" t="s">
+        <v>130</v>
+      </c>
+      <c r="F12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" t="s">
+        <v>144</v>
+      </c>
+      <c r="H12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I12">
+        <v>8.6</v>
+      </c>
+      <c r="J12">
+        <v>7.9</v>
+      </c>
+      <c r="K12" t="s">
+        <v>613</v>
+      </c>
+      <c r="L12" t="s">
+        <v>614</v>
+      </c>
+      <c r="M12" t="s">
+        <v>133</v>
+      </c>
+      <c r="N12" t="s">
+        <v>38</v>
+      </c>
+      <c r="O12">
+        <v>21</v>
+      </c>
+      <c r="P12" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>687</v>
+      </c>
+      <c r="R12">
+        <v>33</v>
+      </c>
+      <c r="S12" t="s">
+        <v>688</v>
+      </c>
+      <c r="T12" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="U12" t="s">
+        <v>66</v>
+      </c>
+      <c r="V12" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W12" t="s">
+        <v>67</v>
+      </c>
+      <c r="X12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>689</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" t="s">
+        <v>691</v>
+      </c>
+      <c r="D13" t="s">
+        <v>153</v>
+      </c>
+      <c r="E13" t="s">
+        <v>130</v>
+      </c>
+      <c r="F13" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" t="s">
+        <v>131</v>
+      </c>
+      <c r="H13" t="s">
+        <v>144</v>
+      </c>
+      <c r="I13">
+        <v>5.6</v>
+      </c>
+      <c r="J13">
+        <v>7.2</v>
+      </c>
+      <c r="K13" t="s">
+        <v>613</v>
+      </c>
+      <c r="L13" t="s">
+        <v>614</v>
+      </c>
+      <c r="M13" t="s">
+        <v>133</v>
+      </c>
+      <c r="N13" t="s">
+        <v>38</v>
+      </c>
+      <c r="O13">
+        <v>9</v>
+      </c>
+      <c r="P13" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>692</v>
+      </c>
+      <c r="R13">
+        <v>52</v>
+      </c>
+      <c r="S13" t="s">
+        <v>693</v>
+      </c>
+      <c r="T13" s="2" t="s">
+        <v>694</v>
+      </c>
+      <c r="U13" t="s">
+        <v>695</v>
+      </c>
+      <c r="V13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W13" t="s">
+        <v>696</v>
+      </c>
+      <c r="X13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>697</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" t="s">
+        <v>699</v>
+      </c>
+      <c r="D14" t="s">
+        <v>162</v>
+      </c>
+      <c r="E14" t="s">
+        <v>130</v>
+      </c>
+      <c r="F14" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" t="s">
+        <v>163</v>
+      </c>
+      <c r="H14" t="s">
+        <v>132</v>
+      </c>
+      <c r="I14">
+        <v>6.6</v>
+      </c>
+      <c r="J14">
+        <v>4.9</v>
+      </c>
+      <c r="K14" t="s">
+        <v>613</v>
+      </c>
+      <c r="L14" t="s">
+        <v>614</v>
+      </c>
+      <c r="M14" t="s">
+        <v>133</v>
+      </c>
+      <c r="N14" t="s">
+        <v>38</v>
+      </c>
+      <c r="O14">
+        <v>18</v>
+      </c>
+      <c r="P14" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>700</v>
+      </c>
+      <c r="R14">
+        <v>22</v>
+      </c>
+      <c r="S14" t="s">
+        <v>362</v>
+      </c>
+      <c r="T14" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="U14" t="s">
+        <v>363</v>
+      </c>
+      <c r="V14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W14" t="s">
+        <v>364</v>
+      </c>
+      <c r="X14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>701</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>703</v>
+      </c>
+      <c r="D15" t="s">
+        <v>172</v>
+      </c>
+      <c r="E15" t="s">
+        <v>130</v>
+      </c>
+      <c r="F15" t="s">
+        <v>60</v>
+      </c>
+      <c r="G15" t="s">
+        <v>131</v>
+      </c>
+      <c r="H15" t="s">
+        <v>163</v>
+      </c>
+      <c r="I15">
+        <v>7.7</v>
+      </c>
+      <c r="J15">
+        <v>7.6</v>
+      </c>
+      <c r="K15" t="s">
+        <v>613</v>
+      </c>
+      <c r="L15" t="s">
+        <v>614</v>
+      </c>
+      <c r="M15" t="s">
+        <v>133</v>
+      </c>
+      <c r="N15" t="s">
+        <v>38</v>
+      </c>
+      <c r="O15">
+        <v>12</v>
+      </c>
+      <c r="P15" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>704</v>
+      </c>
+      <c r="R15">
+        <v>56</v>
+      </c>
+      <c r="S15" t="s">
+        <v>705</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>706</v>
+      </c>
+      <c r="U15" t="s">
+        <v>707</v>
+      </c>
+      <c r="V15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W15" t="s">
+        <v>708</v>
+      </c>
+      <c r="X15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>709</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" t="s">
+        <v>711</v>
+      </c>
+      <c r="D16" t="s">
+        <v>181</v>
+      </c>
+      <c r="E16" t="s">
+        <v>130</v>
+      </c>
+      <c r="F16" t="s">
+        <v>60</v>
+      </c>
+      <c r="G16" t="s">
+        <v>34</v>
+      </c>
+      <c r="H16" t="s">
+        <v>132</v>
+      </c>
+      <c r="I16">
+        <v>11.3</v>
+      </c>
+      <c r="J16">
+        <v>13.3</v>
+      </c>
+      <c r="K16" t="s">
+        <v>613</v>
+      </c>
+      <c r="L16" t="s">
+        <v>614</v>
+      </c>
+      <c r="M16" t="s">
+        <v>133</v>
+      </c>
+      <c r="N16" t="s">
+        <v>38</v>
+      </c>
+      <c r="O16">
+        <v>25</v>
+      </c>
+      <c r="P16" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>712</v>
+      </c>
+      <c r="R16">
+        <v>39</v>
+      </c>
+      <c r="S16" t="s">
+        <v>713</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="U16" t="s">
+        <v>714</v>
+      </c>
+      <c r="V16" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W16" t="s">
+        <v>715</v>
+      </c>
+      <c r="X16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>716</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>718</v>
+      </c>
+      <c r="D17" t="s">
+        <v>190</v>
+      </c>
+      <c r="E17" t="s">
+        <v>191</v>
+      </c>
+      <c r="F17" t="s">
+        <v>32</v>
+      </c>
+      <c r="G17" t="s">
+        <v>110</v>
+      </c>
+      <c r="H17" t="s">
+        <v>192</v>
+      </c>
+      <c r="I17">
+        <v>9.8</v>
+      </c>
+      <c r="J17">
+        <v>9.8</v>
+      </c>
+      <c r="K17" t="s">
+        <v>613</v>
+      </c>
+      <c r="L17" t="s">
+        <v>614</v>
+      </c>
+      <c r="M17" t="s">
+        <v>193</v>
+      </c>
+      <c r="N17" t="s">
+        <v>38</v>
+      </c>
+      <c r="O17">
+        <v>28</v>
+      </c>
+      <c r="P17" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>551</v>
+      </c>
+      <c r="R17">
+        <v>28</v>
+      </c>
+      <c r="S17" t="s">
+        <v>719</v>
+      </c>
+      <c r="T17" t="s">
+        <v>113</v>
+      </c>
+      <c r="U17" t="s">
+        <v>114</v>
+      </c>
+      <c r="V17" t="s">
+        <v>115</v>
+      </c>
+      <c r="W17" t="s">
+        <v>116</v>
+      </c>
+      <c r="X17" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>720</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" t="s">
+        <v>722</v>
+      </c>
+      <c r="D18" t="s">
+        <v>202</v>
+      </c>
+      <c r="E18" t="s">
+        <v>191</v>
+      </c>
+      <c r="F18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" t="s">
+        <v>203</v>
+      </c>
+      <c r="H18" t="s">
+        <v>192</v>
+      </c>
+      <c r="I18">
+        <v>4.4</v>
+      </c>
+      <c r="J18">
+        <v>4.4</v>
+      </c>
+      <c r="K18" t="s">
+        <v>613</v>
+      </c>
+      <c r="L18" t="s">
+        <v>614</v>
+      </c>
+      <c r="M18" t="s">
+        <v>193</v>
+      </c>
+      <c r="N18" t="s">
+        <v>38</v>
+      </c>
+      <c r="O18">
+        <v>17</v>
+      </c>
+      <c r="P18" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>723</v>
+      </c>
+      <c r="R18">
+        <v>11</v>
+      </c>
+      <c r="S18" t="s">
+        <v>724</v>
+      </c>
+      <c r="T18" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="U18" t="s">
+        <v>725</v>
+      </c>
+      <c r="V18" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="W18" t="s">
+        <v>726</v>
+      </c>
+      <c r="X18" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>727</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>729</v>
+      </c>
+      <c r="D19" t="s">
+        <v>210</v>
+      </c>
+      <c r="E19" t="s">
+        <v>191</v>
+      </c>
+      <c r="F19" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" t="s">
+        <v>110</v>
+      </c>
+      <c r="H19" t="s">
+        <v>211</v>
+      </c>
+      <c r="I19">
+        <v>8.9</v>
+      </c>
+      <c r="J19">
+        <v>8.8</v>
+      </c>
+      <c r="K19" t="s">
+        <v>613</v>
+      </c>
+      <c r="L19" t="s">
+        <v>614</v>
+      </c>
+      <c r="M19" t="s">
+        <v>193</v>
+      </c>
+      <c r="N19" t="s">
+        <v>38</v>
+      </c>
+      <c r="O19">
+        <v>23</v>
+      </c>
+      <c r="P19" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>565</v>
+      </c>
+      <c r="R19">
+        <v>26</v>
+      </c>
+      <c r="S19" t="s">
+        <v>730</v>
+      </c>
+      <c r="T19" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U19" t="s">
+        <v>241</v>
+      </c>
+      <c r="V19" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W19" t="s">
+        <v>731</v>
+      </c>
+      <c r="X19" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>732</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" t="s">
+        <v>734</v>
+      </c>
+      <c r="D20" t="s">
+        <v>219</v>
+      </c>
+      <c r="E20" t="s">
+        <v>220</v>
+      </c>
+      <c r="F20" t="s">
+        <v>32</v>
+      </c>
+      <c r="G20" t="s">
+        <v>221</v>
+      </c>
+      <c r="H20" t="s">
+        <v>222</v>
+      </c>
+      <c r="I20">
+        <v>7.9</v>
+      </c>
+      <c r="J20">
+        <v>7.8</v>
+      </c>
+      <c r="K20" t="s">
+        <v>613</v>
+      </c>
+      <c r="L20" t="s">
+        <v>614</v>
+      </c>
+      <c r="M20" t="s">
+        <v>223</v>
+      </c>
+      <c r="N20" t="s">
+        <v>38</v>
+      </c>
+      <c r="O20">
+        <v>17</v>
+      </c>
+      <c r="P20" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>735</v>
+      </c>
+      <c r="R20">
+        <v>29</v>
+      </c>
+      <c r="S20" t="s">
+        <v>736</v>
+      </c>
+      <c r="T20" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="U20" t="s">
+        <v>737</v>
+      </c>
+      <c r="V20" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W20" t="s">
+        <v>738</v>
+      </c>
+      <c r="X20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>739</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C21" t="s">
+        <v>741</v>
+      </c>
+      <c r="D21" t="s">
+        <v>229</v>
+      </c>
+      <c r="E21" t="s">
+        <v>220</v>
+      </c>
+      <c r="F21" t="s">
+        <v>60</v>
+      </c>
+      <c r="G21" t="s">
+        <v>230</v>
+      </c>
+      <c r="H21" t="s">
+        <v>222</v>
+      </c>
+      <c r="I21">
+        <v>3.7</v>
+      </c>
+      <c r="J21">
+        <v>3.7</v>
+      </c>
+      <c r="K21" t="s">
+        <v>613</v>
+      </c>
+      <c r="L21" t="s">
+        <v>614</v>
+      </c>
+      <c r="M21" t="s">
+        <v>223</v>
+      </c>
+      <c r="N21" t="s">
+        <v>38</v>
+      </c>
+      <c r="O21">
+        <v>9</v>
+      </c>
+      <c r="P21" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>742</v>
+      </c>
+      <c r="R21">
+        <v>16</v>
+      </c>
+      <c r="S21" t="s">
+        <v>743</v>
+      </c>
+      <c r="T21" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="U21" t="s">
+        <v>744</v>
+      </c>
+      <c r="V21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W21" t="s">
+        <v>745</v>
+      </c>
+      <c r="X21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>746</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" t="s">
+        <v>748</v>
+      </c>
+      <c r="D22" t="s">
+        <v>238</v>
+      </c>
+      <c r="E22" t="s">
+        <v>220</v>
+      </c>
+      <c r="F22" t="s">
+        <v>60</v>
+      </c>
+      <c r="G22" t="s">
+        <v>221</v>
+      </c>
+      <c r="H22" t="s">
+        <v>230</v>
+      </c>
+      <c r="I22">
+        <v>4.2</v>
+      </c>
+      <c r="J22">
+        <v>4.1</v>
+      </c>
+      <c r="K22" t="s">
+        <v>613</v>
+      </c>
+      <c r="L22" t="s">
+        <v>614</v>
+      </c>
+      <c r="M22" t="s">
+        <v>223</v>
+      </c>
+      <c r="N22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O22">
+        <v>8</v>
+      </c>
+      <c r="P22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>749</v>
+      </c>
+      <c r="R22">
+        <v>13</v>
+      </c>
+      <c r="S22" t="s">
+        <v>586</v>
+      </c>
+      <c r="T22" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="U22" t="s">
+        <v>750</v>
+      </c>
+      <c r="V22" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W22" t="s">
+        <v>751</v>
+      </c>
+      <c r="X22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>752</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C23" t="s">
+        <v>754</v>
+      </c>
+      <c r="D23" t="s">
+        <v>246</v>
+      </c>
+      <c r="E23" t="s">
+        <v>220</v>
+      </c>
+      <c r="F23" t="s">
+        <v>60</v>
+      </c>
+      <c r="G23" t="s">
+        <v>221</v>
+      </c>
+      <c r="H23" t="s">
+        <v>247</v>
+      </c>
+      <c r="I23">
+        <v>6.6</v>
+      </c>
+      <c r="J23">
+        <v>6.5</v>
+      </c>
+      <c r="K23" t="s">
+        <v>613</v>
+      </c>
+      <c r="L23" t="s">
+        <v>614</v>
+      </c>
+      <c r="M23" t="s">
+        <v>223</v>
+      </c>
+      <c r="N23" t="s">
+        <v>38</v>
+      </c>
+      <c r="O23">
+        <v>14</v>
+      </c>
+      <c r="P23" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>755</v>
+      </c>
+      <c r="R23">
+        <v>22</v>
+      </c>
+      <c r="S23" t="s">
+        <v>756</v>
+      </c>
+      <c r="T23" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="U23" t="s">
+        <v>66</v>
+      </c>
+      <c r="V23" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W23" t="s">
+        <v>67</v>
+      </c>
+      <c r="X23" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>757</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>27</v>
+      </c>
+      <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" t="s">
+        <v>759</v>
+      </c>
+      <c r="D24" t="s">
+        <v>255</v>
+      </c>
+      <c r="E24" t="s">
+        <v>220</v>
+      </c>
+      <c r="F24" t="s">
+        <v>60</v>
+      </c>
+      <c r="G24" t="s">
+        <v>230</v>
+      </c>
+      <c r="H24" t="s">
+        <v>247</v>
+      </c>
+      <c r="I24">
+        <v>2.4</v>
+      </c>
+      <c r="J24">
+        <v>2.4</v>
+      </c>
+      <c r="K24" t="s">
+        <v>613</v>
+      </c>
+      <c r="L24" t="s">
+        <v>614</v>
+      </c>
+      <c r="M24" t="s">
+        <v>223</v>
+      </c>
+      <c r="N24" t="s">
+        <v>38</v>
+      </c>
+      <c r="O24">
+        <v>6</v>
+      </c>
+      <c r="P24" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>760</v>
+      </c>
+      <c r="R24">
+        <v>9</v>
+      </c>
+      <c r="S24" t="s">
+        <v>429</v>
+      </c>
+      <c r="T24" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U24" t="s">
+        <v>430</v>
+      </c>
+      <c r="V24" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W24" t="s">
+        <v>431</v>
+      </c>
+      <c r="X24" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>761</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>763</v>
+      </c>
+      <c r="D25" t="s">
+        <v>263</v>
+      </c>
+      <c r="E25" t="s">
+        <v>220</v>
+      </c>
+      <c r="F25" t="s">
+        <v>60</v>
+      </c>
+      <c r="G25" t="s">
+        <v>247</v>
+      </c>
+      <c r="H25" t="s">
+        <v>222</v>
+      </c>
+      <c r="I25">
+        <v>1.3</v>
+      </c>
+      <c r="J25">
+        <v>1.3</v>
+      </c>
+      <c r="K25" t="s">
+        <v>613</v>
+      </c>
+      <c r="L25" t="s">
+        <v>614</v>
+      </c>
+      <c r="M25" t="s">
+        <v>223</v>
+      </c>
+      <c r="N25" t="s">
+        <v>38</v>
+      </c>
+      <c r="O25">
+        <v>3</v>
+      </c>
+      <c r="P25" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>764</v>
+      </c>
+      <c r="R25">
+        <v>6</v>
+      </c>
+      <c r="S25" t="s">
+        <v>765</v>
+      </c>
+      <c r="T25" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U25" t="s">
+        <v>766</v>
+      </c>
+      <c r="V25" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="W25" t="s">
+        <v>767</v>
+      </c>
+      <c r="X25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>768</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>769</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AA1"/>
+  <hyperlinks>
+    <hyperlink ref="X2" r:id="rId1"/>
+    <hyperlink ref="Y2" r:id="rId2"/>
+    <hyperlink ref="X3" r:id="rId3"/>
+    <hyperlink ref="Y3" r:id="rId4"/>
+    <hyperlink ref="X4" r:id="rId5"/>
+    <hyperlink ref="Y4" r:id="rId6"/>
+    <hyperlink ref="X5" r:id="rId7"/>
+    <hyperlink ref="Y5" r:id="rId8"/>
+    <hyperlink ref="X6" r:id="rId9"/>
+    <hyperlink ref="Y6" r:id="rId10"/>
+    <hyperlink ref="X7" r:id="rId11"/>
+    <hyperlink ref="Y7" r:id="rId12"/>
+    <hyperlink ref="X8" r:id="rId13"/>
+    <hyperlink ref="Y8" r:id="rId14"/>
+    <hyperlink ref="X9" r:id="rId15"/>
+    <hyperlink ref="Y9" r:id="rId16"/>
+    <hyperlink ref="X10" r:id="rId17"/>
+    <hyperlink ref="Y10" r:id="rId18"/>
+    <hyperlink ref="X11" r:id="rId19"/>
+    <hyperlink ref="Y11" r:id="rId20"/>
+    <hyperlink ref="X12" r:id="rId21"/>
+    <hyperlink ref="Y12" r:id="rId22"/>
+    <hyperlink ref="X13" r:id="rId23"/>
+    <hyperlink ref="Y13" r:id="rId24"/>
+    <hyperlink ref="X14" r:id="rId25"/>
+    <hyperlink ref="Y14" r:id="rId26"/>
+    <hyperlink ref="X15" r:id="rId27"/>
+    <hyperlink ref="Y15" r:id="rId28"/>
+    <hyperlink ref="X16" r:id="rId29"/>
+    <hyperlink ref="Y16" r:id="rId30"/>
+    <hyperlink ref="X17" r:id="rId31"/>
+    <hyperlink ref="Y17" r:id="rId32"/>
+    <hyperlink ref="X18" r:id="rId33"/>
+    <hyperlink ref="Y18" r:id="rId34"/>
+    <hyperlink ref="X19" r:id="rId35"/>
+    <hyperlink ref="Y19" r:id="rId36"/>
+    <hyperlink ref="X20" r:id="rId37"/>
+    <hyperlink ref="Y20" r:id="rId38"/>
+    <hyperlink ref="X21" r:id="rId39"/>
+    <hyperlink ref="Y21" r:id="rId40"/>
+    <hyperlink ref="X22" r:id="rId41"/>
+    <hyperlink ref="Y22" r:id="rId42"/>
+    <hyperlink ref="X23" r:id="rId43"/>
+    <hyperlink ref="Y23" r:id="rId44"/>
+    <hyperlink ref="X24" r:id="rId45"/>
+    <hyperlink ref="Y24" r:id="rId46"/>
+    <hyperlink ref="X25" r:id="rId47"/>
+    <hyperlink ref="Y25" r:id="rId48"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:AP25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:42" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>3</v>
       </c>
@@ -8774,88 +11413,115 @@
         <v>9</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>612</v>
+        <v>770</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>613</v>
+        <v>771</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>614</v>
+        <v>772</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>615</v>
+        <v>773</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>616</v>
+        <v>774</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>617</v>
+        <v>775</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>618</v>
+        <v>776</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>619</v>
+        <v>777</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>620</v>
+        <v>778</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>621</v>
+        <v>779</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>622</v>
+        <v>780</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>623</v>
+        <v>781</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>624</v>
+        <v>782</v>
       </c>
       <c r="T1" s="4" t="s">
-        <v>625</v>
+        <v>783</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>626</v>
+        <v>784</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>627</v>
+        <v>785</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>628</v>
+        <v>786</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>629</v>
+        <v>787</v>
       </c>
       <c r="Y1" s="4" t="s">
-        <v>630</v>
+        <v>788</v>
       </c>
       <c r="Z1" s="4" t="s">
-        <v>631</v>
+        <v>789</v>
       </c>
       <c r="AA1" s="4" t="s">
-        <v>632</v>
+        <v>790</v>
       </c>
       <c r="AB1" s="4" t="s">
-        <v>633</v>
+        <v>791</v>
       </c>
       <c r="AC1" s="4" t="s">
-        <v>634</v>
+        <v>792</v>
       </c>
       <c r="AD1" s="4" t="s">
-        <v>635</v>
+        <v>793</v>
       </c>
       <c r="AE1" s="4" t="s">
-        <v>636</v>
+        <v>794</v>
       </c>
       <c r="AF1" s="4" t="s">
-        <v>637</v>
+        <v>795</v>
       </c>
       <c r="AG1" s="4" t="s">
-        <v>638</v>
+        <v>796</v>
+      </c>
+      <c r="AH1" s="4" t="s">
+        <v>797</v>
+      </c>
+      <c r="AI1" s="4" t="s">
+        <v>798</v>
+      </c>
+      <c r="AJ1" s="4" t="s">
+        <v>799</v>
+      </c>
+      <c r="AK1" s="4" t="s">
+        <v>800</v>
+      </c>
+      <c r="AL1" s="4" t="s">
+        <v>801</v>
+      </c>
+      <c r="AM1" s="4" t="s">
+        <v>802</v>
+      </c>
+      <c r="AN1" s="4" t="s">
+        <v>803</v>
+      </c>
+      <c r="AO1" s="4" t="s">
+        <v>804</v>
+      </c>
+      <c r="AP1" s="4" t="s">
+        <v>805</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -8955,8 +11621,35 @@
       <c r="AG2" t="s">
         <v>446</v>
       </c>
+      <c r="AH2" t="s">
+        <v>612</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK2">
+        <v>28</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>615</v>
+      </c>
+      <c r="AN2">
+        <v>52</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>618</v>
+      </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -9056,8 +11749,35 @@
       <c r="AG3" t="s">
         <v>454</v>
       </c>
+      <c r="AH3" t="s">
+        <v>621</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK3">
+        <v>29</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>622</v>
+      </c>
+      <c r="AN3">
+        <v>68</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP3" t="s">
+        <v>626</v>
+      </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>59</v>
       </c>
@@ -9143,7 +11863,7 @@
         <v>54</v>
       </c>
       <c r="AC4" t="s">
-        <v>639</v>
+        <v>806</v>
       </c>
       <c r="AD4" t="s">
         <v>458</v>
@@ -9157,8 +11877,35 @@
       <c r="AG4" t="s">
         <v>462</v>
       </c>
+      <c r="AH4" t="s">
+        <v>629</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK4">
+        <v>8</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>630</v>
+      </c>
+      <c r="AN4">
+        <v>18</v>
+      </c>
+      <c r="AO4" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP4" t="s">
+        <v>632</v>
+      </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>71</v>
       </c>
@@ -9258,8 +12005,35 @@
       <c r="AG5" t="s">
         <v>470</v>
       </c>
+      <c r="AH5" t="s">
+        <v>635</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK5">
+        <v>11</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>636</v>
+      </c>
+      <c r="AN5">
+        <v>31</v>
+      </c>
+      <c r="AO5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP5" t="s">
+        <v>640</v>
+      </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>80</v>
       </c>
@@ -9359,8 +12133,35 @@
       <c r="AG6" t="s">
         <v>478</v>
       </c>
+      <c r="AH6" t="s">
+        <v>643</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK6">
+        <v>11</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM6" t="s">
+        <v>644</v>
+      </c>
+      <c r="AN6">
+        <v>28</v>
+      </c>
+      <c r="AO6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP6" t="s">
+        <v>648</v>
+      </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>90</v>
       </c>
@@ -9460,8 +12261,35 @@
       <c r="AG7" t="s">
         <v>484</v>
       </c>
+      <c r="AH7" t="s">
+        <v>651</v>
+      </c>
+      <c r="AI7" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK7">
+        <v>12</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM7" t="s">
+        <v>652</v>
+      </c>
+      <c r="AN7">
+        <v>26</v>
+      </c>
+      <c r="AO7" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP7" t="s">
+        <v>454</v>
+      </c>
     </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>99</v>
       </c>
@@ -9561,8 +12389,35 @@
       <c r="AG8" t="s">
         <v>491</v>
       </c>
+      <c r="AH8" t="s">
+        <v>656</v>
+      </c>
+      <c r="AI8" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ8" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK8">
+        <v>18</v>
+      </c>
+      <c r="AL8" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM8" t="s">
+        <v>657</v>
+      </c>
+      <c r="AN8">
+        <v>40</v>
+      </c>
+      <c r="AO8" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP8" t="s">
+        <v>660</v>
+      </c>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>109</v>
       </c>
@@ -9662,8 +12517,35 @@
       <c r="AG9" t="s">
         <v>498</v>
       </c>
+      <c r="AH9" t="s">
+        <v>663</v>
+      </c>
+      <c r="AI9" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ9" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK9">
+        <v>15</v>
+      </c>
+      <c r="AL9" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM9" t="s">
+        <v>664</v>
+      </c>
+      <c r="AN9">
+        <v>32</v>
+      </c>
+      <c r="AO9" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP9" t="s">
+        <v>667</v>
+      </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>120</v>
       </c>
@@ -9763,8 +12645,35 @@
       <c r="AG10" t="s">
         <v>506</v>
       </c>
+      <c r="AH10" t="s">
+        <v>670</v>
+      </c>
+      <c r="AI10" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ10" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK10">
+        <v>16</v>
+      </c>
+      <c r="AL10" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM10" t="s">
+        <v>671</v>
+      </c>
+      <c r="AN10">
+        <v>46</v>
+      </c>
+      <c r="AO10" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP10" t="s">
+        <v>675</v>
+      </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>129</v>
       </c>
@@ -9864,8 +12773,35 @@
       <c r="AG11" t="s">
         <v>513</v>
       </c>
+      <c r="AH11" t="s">
+        <v>678</v>
+      </c>
+      <c r="AI11" t="s">
+        <v>133</v>
+      </c>
+      <c r="AJ11" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK11">
+        <v>30</v>
+      </c>
+      <c r="AL11" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM11" t="s">
+        <v>679</v>
+      </c>
+      <c r="AN11">
+        <v>66</v>
+      </c>
+      <c r="AO11" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP11" t="s">
+        <v>683</v>
+      </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>143</v>
       </c>
@@ -9965,8 +12901,35 @@
       <c r="AG12" t="s">
         <v>520</v>
       </c>
+      <c r="AH12" t="s">
+        <v>686</v>
+      </c>
+      <c r="AI12" t="s">
+        <v>133</v>
+      </c>
+      <c r="AJ12" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK12">
+        <v>21</v>
+      </c>
+      <c r="AL12" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM12" t="s">
+        <v>687</v>
+      </c>
+      <c r="AN12">
+        <v>33</v>
+      </c>
+      <c r="AO12" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP12" t="s">
+        <v>67</v>
+      </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>153</v>
       </c>
@@ -10066,8 +13029,35 @@
       <c r="AG13" t="s">
         <v>528</v>
       </c>
+      <c r="AH13" t="s">
+        <v>691</v>
+      </c>
+      <c r="AI13" t="s">
+        <v>133</v>
+      </c>
+      <c r="AJ13" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK13">
+        <v>9</v>
+      </c>
+      <c r="AL13" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM13" t="s">
+        <v>692</v>
+      </c>
+      <c r="AN13">
+        <v>52</v>
+      </c>
+      <c r="AO13" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP13" t="s">
+        <v>696</v>
+      </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>162</v>
       </c>
@@ -10167,8 +13157,35 @@
       <c r="AG14" t="s">
         <v>116</v>
       </c>
+      <c r="AH14" t="s">
+        <v>699</v>
+      </c>
+      <c r="AI14" t="s">
+        <v>133</v>
+      </c>
+      <c r="AJ14" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK14">
+        <v>18</v>
+      </c>
+      <c r="AL14" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM14" t="s">
+        <v>700</v>
+      </c>
+      <c r="AN14">
+        <v>22</v>
+      </c>
+      <c r="AO14" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP14" t="s">
+        <v>364</v>
+      </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>172</v>
       </c>
@@ -10268,8 +13285,35 @@
       <c r="AG15" t="s">
         <v>540</v>
       </c>
+      <c r="AH15" t="s">
+        <v>703</v>
+      </c>
+      <c r="AI15" t="s">
+        <v>133</v>
+      </c>
+      <c r="AJ15" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK15">
+        <v>12</v>
+      </c>
+      <c r="AL15" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM15" t="s">
+        <v>704</v>
+      </c>
+      <c r="AN15">
+        <v>56</v>
+      </c>
+      <c r="AO15" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP15" t="s">
+        <v>708</v>
+      </c>
     </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>181</v>
       </c>
@@ -10369,8 +13413,35 @@
       <c r="AG16" t="s">
         <v>547</v>
       </c>
+      <c r="AH16" t="s">
+        <v>711</v>
+      </c>
+      <c r="AI16" t="s">
+        <v>133</v>
+      </c>
+      <c r="AJ16" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK16">
+        <v>25</v>
+      </c>
+      <c r="AL16" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM16" t="s">
+        <v>712</v>
+      </c>
+      <c r="AN16">
+        <v>39</v>
+      </c>
+      <c r="AO16" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP16" t="s">
+        <v>715</v>
+      </c>
     </row>
-    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>190</v>
       </c>
@@ -10470,8 +13541,35 @@
       <c r="AG17" t="s">
         <v>554</v>
       </c>
+      <c r="AH17" t="s">
+        <v>718</v>
+      </c>
+      <c r="AI17" t="s">
+        <v>193</v>
+      </c>
+      <c r="AJ17" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK17">
+        <v>28</v>
+      </c>
+      <c r="AL17" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM17" t="s">
+        <v>551</v>
+      </c>
+      <c r="AN17">
+        <v>28</v>
+      </c>
+      <c r="AO17" t="s">
+        <v>115</v>
+      </c>
+      <c r="AP17" t="s">
+        <v>116</v>
+      </c>
     </row>
-    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>202</v>
       </c>
@@ -10571,8 +13669,35 @@
       <c r="AG18" t="s">
         <v>561</v>
       </c>
+      <c r="AH18" t="s">
+        <v>722</v>
+      </c>
+      <c r="AI18" t="s">
+        <v>193</v>
+      </c>
+      <c r="AJ18" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK18">
+        <v>17</v>
+      </c>
+      <c r="AL18" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM18" t="s">
+        <v>723</v>
+      </c>
+      <c r="AN18">
+        <v>11</v>
+      </c>
+      <c r="AO18" t="s">
+        <v>138</v>
+      </c>
+      <c r="AP18" t="s">
+        <v>726</v>
+      </c>
     </row>
-    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>210</v>
       </c>
@@ -10672,8 +13797,35 @@
       <c r="AG19" t="s">
         <v>568</v>
       </c>
+      <c r="AH19" t="s">
+        <v>729</v>
+      </c>
+      <c r="AI19" t="s">
+        <v>193</v>
+      </c>
+      <c r="AJ19" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK19">
+        <v>23</v>
+      </c>
+      <c r="AL19" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM19" t="s">
+        <v>565</v>
+      </c>
+      <c r="AN19">
+        <v>26</v>
+      </c>
+      <c r="AO19" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP19" t="s">
+        <v>731</v>
+      </c>
     </row>
-    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>219</v>
       </c>
@@ -10773,8 +13925,35 @@
       <c r="AG20" t="s">
         <v>498</v>
       </c>
+      <c r="AH20" t="s">
+        <v>734</v>
+      </c>
+      <c r="AI20" t="s">
+        <v>223</v>
+      </c>
+      <c r="AJ20" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK20">
+        <v>17</v>
+      </c>
+      <c r="AL20" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM20" t="s">
+        <v>735</v>
+      </c>
+      <c r="AN20">
+        <v>29</v>
+      </c>
+      <c r="AO20" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP20" t="s">
+        <v>738</v>
+      </c>
     </row>
-    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>229</v>
       </c>
@@ -10860,7 +14039,7 @@
         <v>51</v>
       </c>
       <c r="AC21" t="s">
-        <v>639</v>
+        <v>806</v>
       </c>
       <c r="AD21" t="s">
         <v>577</v>
@@ -10874,8 +14053,35 @@
       <c r="AG21" t="s">
         <v>581</v>
       </c>
+      <c r="AH21" t="s">
+        <v>741</v>
+      </c>
+      <c r="AI21" t="s">
+        <v>223</v>
+      </c>
+      <c r="AJ21" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK21">
+        <v>9</v>
+      </c>
+      <c r="AL21" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM21" t="s">
+        <v>742</v>
+      </c>
+      <c r="AN21">
+        <v>16</v>
+      </c>
+      <c r="AO21" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP21" t="s">
+        <v>745</v>
+      </c>
     </row>
-    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>238</v>
       </c>
@@ -10961,7 +14167,7 @@
         <v>57</v>
       </c>
       <c r="AC22" t="s">
-        <v>639</v>
+        <v>806</v>
       </c>
       <c r="AD22" t="s">
         <v>585</v>
@@ -10975,8 +14181,35 @@
       <c r="AG22" t="s">
         <v>589</v>
       </c>
+      <c r="AH22" t="s">
+        <v>748</v>
+      </c>
+      <c r="AI22" t="s">
+        <v>223</v>
+      </c>
+      <c r="AJ22" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK22">
+        <v>8</v>
+      </c>
+      <c r="AL22" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM22" t="s">
+        <v>749</v>
+      </c>
+      <c r="AN22">
+        <v>13</v>
+      </c>
+      <c r="AO22" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP22" t="s">
+        <v>751</v>
+      </c>
     </row>
-    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>246</v>
       </c>
@@ -11076,8 +14309,35 @@
       <c r="AG23" t="s">
         <v>424</v>
       </c>
+      <c r="AH23" t="s">
+        <v>754</v>
+      </c>
+      <c r="AI23" t="s">
+        <v>223</v>
+      </c>
+      <c r="AJ23" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK23">
+        <v>14</v>
+      </c>
+      <c r="AL23" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM23" t="s">
+        <v>755</v>
+      </c>
+      <c r="AN23">
+        <v>22</v>
+      </c>
+      <c r="AO23" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP23" t="s">
+        <v>67</v>
+      </c>
     </row>
-    <row r="24" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>255</v>
       </c>
@@ -11163,7 +14423,7 @@
         <v>33</v>
       </c>
       <c r="AC24" t="s">
-        <v>639</v>
+        <v>806</v>
       </c>
       <c r="AD24" t="s">
         <v>597</v>
@@ -11177,8 +14437,35 @@
       <c r="AG24" t="s">
         <v>601</v>
       </c>
+      <c r="AH24" t="s">
+        <v>759</v>
+      </c>
+      <c r="AI24" t="s">
+        <v>223</v>
+      </c>
+      <c r="AJ24" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK24">
+        <v>6</v>
+      </c>
+      <c r="AL24" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM24" t="s">
+        <v>760</v>
+      </c>
+      <c r="AN24">
+        <v>9</v>
+      </c>
+      <c r="AO24" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP24" t="s">
+        <v>431</v>
+      </c>
     </row>
-    <row r="25" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>263</v>
       </c>
@@ -11264,7 +14551,7 @@
         <v>18</v>
       </c>
       <c r="AC25" t="s">
-        <v>639</v>
+        <v>806</v>
       </c>
       <c r="AD25" t="s">
         <v>605</v>
@@ -11278,9 +14565,36 @@
       <c r="AG25" t="s">
         <v>609</v>
       </c>
+      <c r="AH25" t="s">
+        <v>763</v>
+      </c>
+      <c r="AI25" t="s">
+        <v>223</v>
+      </c>
+      <c r="AJ25" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK25">
+        <v>3</v>
+      </c>
+      <c r="AL25" t="s">
+        <v>39</v>
+      </c>
+      <c r="AM25" t="s">
+        <v>764</v>
+      </c>
+      <c r="AN25">
+        <v>6</v>
+      </c>
+      <c r="AO25" t="s">
+        <v>39</v>
+      </c>
+      <c r="AP25" t="s">
+        <v>767</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AG1"/>
+  <autoFilter ref="A1:AP1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>